<commit_message>
split/rotate calendar view to minimixe vertical size
</commit_message>
<xml_diff>
--- a/src/stp/database/localization.xlsx
+++ b/src/stp/database/localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7505B6D6-844A-A947-BACC-5F267A636214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD23A79-014A-4A40-8E6D-56533CFAB06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Competition" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3434" uniqueCount="2222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3462" uniqueCount="2227">
   <si>
     <t>key</t>
   </si>
@@ -6661,9 +6661,6 @@
     <t>zh_Hant</t>
   </si>
   <si>
-    <t>en_GB</t>
-  </si>
-  <si>
     <t>Dieciseisavos de final</t>
   </si>
   <si>
@@ -6695,6 +6692,24 @@
   </si>
   <si>
     <t>Nordamerica</t>
+  </si>
+  <si>
+    <t>en_alt</t>
+  </si>
+  <si>
+    <t>ja_alt</t>
+  </si>
+  <si>
+    <t>NotoSansCJKjp-Light.otf</t>
+  </si>
+  <si>
+    <t>NotoSansCJKjp-Regular.otf</t>
+  </si>
+  <si>
+    <t>NotoSansCJKjp-Bold.otf</t>
+  </si>
+  <si>
+    <t>calendar.day-of-week-broken</t>
   </si>
 </sst>
 </file>
@@ -6772,18 +6787,19 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}" name="Table10" displayName="Table10" ref="A1:N27" totalsRowShown="0">
-  <autoFilter ref="A1:N27" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}" name="Table10" displayName="Table10" ref="A1:O28" totalsRowShown="0">
+  <autoFilter ref="A1:O28" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}"/>
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{ED366778-7374-0B4D-B3D7-3A1347569CE0}" name="key"/>
     <tableColumn id="2" xr3:uid="{80E7518A-3634-0641-9EC4-DD7EB1B380BB}" name="en"/>
-    <tableColumn id="3" xr3:uid="{FE7E56C3-4451-AE4D-B1AF-92EFC944B7F5}" name="en_GB"/>
+    <tableColumn id="3" xr3:uid="{FE7E56C3-4451-AE4D-B1AF-92EFC944B7F5}" name="en_alt"/>
     <tableColumn id="4" xr3:uid="{5EC5DC67-5B41-8A4F-95A2-607E7726E4C3}" name="es"/>
     <tableColumn id="5" xr3:uid="{D551C02C-16D0-3B4E-B610-0C030C46992D}" name="it"/>
     <tableColumn id="6" xr3:uid="{A53D972F-0712-3B43-ADB6-55DCB6B64D5E}" name="fr"/>
     <tableColumn id="7" xr3:uid="{41CEB9F8-F4C9-F040-92D6-2BF6B13D0CB3}" name="de"/>
     <tableColumn id="8" xr3:uid="{FD602427-FAAB-154F-8194-4587249051BC}" name="nl"/>
-    <tableColumn id="9" xr3:uid="{438BCE97-8A7A-EC4A-B263-6ECA8C0D3BB1}" name="ja"/>
+    <tableColumn id="15" xr3:uid="{B1CB1C0C-D5DA-524B-BC41-F9230EA4F8AA}" name="ja"/>
+    <tableColumn id="9" xr3:uid="{438BCE97-8A7A-EC4A-B263-6ECA8C0D3BB1}" name="ja_alt"/>
     <tableColumn id="10" xr3:uid="{EAF98D58-A095-9C4F-918D-34BD7D07524B}" name="fa"/>
     <tableColumn id="11" xr3:uid="{45987AA2-44FB-784C-93AE-022FD26892F7}" name="pt"/>
     <tableColumn id="12" xr3:uid="{AF687974-098A-8941-875B-EAFF0D8C9E19}" name="ko"/>
@@ -7513,23 +7529,24 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="4.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7537,7 +7554,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2210</v>
+        <v>2221</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -7558,22 +7575,25 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
+        <v>2222</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>2208</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>2209</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2148</v>
       </c>
@@ -7584,76 +7604,85 @@
         <v>2150</v>
       </c>
       <c r="I2" t="s">
+        <v>2223</v>
+      </c>
+      <c r="J2" t="s">
         <v>2151</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>2152</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>2198</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>2201</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>2204</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>2226</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2160</v>
+      </c>
+      <c r="I3" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J3" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K3" t="s">
+        <v>2160</v>
+      </c>
+      <c r="M3" t="s">
+        <v>2200</v>
+      </c>
+      <c r="N3" t="s">
+        <v>2203</v>
+      </c>
+      <c r="O3" t="s">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>2153</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>2149</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>2150</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I4" t="s">
+        <v>2223</v>
+      </c>
+      <c r="J4" t="s">
         <v>2151</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K4" t="s">
         <v>2152</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M4" t="s">
         <v>2198</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N4" t="s">
         <v>2201</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O4" t="s">
         <v>2204</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>2154</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2155</v>
-      </c>
-      <c r="C4" t="s">
-        <v>2152</v>
-      </c>
-      <c r="I4" t="s">
-        <v>2156</v>
-      </c>
-      <c r="J4" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L4" t="s">
-        <v>2199</v>
-      </c>
-      <c r="M4" t="s">
-        <v>2202</v>
-      </c>
-      <c r="N4" t="s">
-        <v>2205</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>2157</v>
       </c>
       <c r="B5" t="s">
         <v>2155</v>
@@ -7662,50 +7691,56 @@
         <v>2152</v>
       </c>
       <c r="I5" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J5" t="s">
         <v>2156</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>2152</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>2199</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>2202</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>2205</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2152</v>
+      </c>
+      <c r="I6" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J6" t="s">
+        <v>2156</v>
+      </c>
+      <c r="K6" t="s">
+        <v>2152</v>
+      </c>
+      <c r="M6" t="s">
+        <v>2199</v>
+      </c>
+      <c r="N6" t="s">
+        <v>2202</v>
+      </c>
+      <c r="O6" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>2158</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2159</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2160</v>
-      </c>
-      <c r="I6" t="s">
-        <v>2161</v>
-      </c>
-      <c r="J6" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L6" t="s">
-        <v>2200</v>
-      </c>
-      <c r="M6" t="s">
-        <v>2203</v>
-      </c>
-      <c r="N6" t="s">
-        <v>2206</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>2162</v>
       </c>
       <c r="B7" t="s">
         <v>2159</v>
@@ -7714,280 +7749,307 @@
         <v>2160</v>
       </c>
       <c r="I7" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J7" t="s">
         <v>2161</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>2160</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>2200</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>2203</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>2206</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2160</v>
+      </c>
+      <c r="I8" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J8" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K8" t="s">
+        <v>2160</v>
+      </c>
+      <c r="M8" t="s">
+        <v>2200</v>
+      </c>
+      <c r="N8" t="s">
+        <v>2203</v>
+      </c>
+      <c r="O8" t="s">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>2163</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>2164</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>2152</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I9" t="s">
+        <v>2223</v>
+      </c>
+      <c r="J9" t="s">
         <v>2151</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K9" t="s">
         <v>2152</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M9" t="s">
         <v>2198</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N9" t="s">
         <v>2201</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O9" t="s">
         <v>2204</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>2165</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>2159</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>2160</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I10" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J10" t="s">
         <v>2161</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K10" t="s">
         <v>2160</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M10" t="s">
         <v>2200</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N10" t="s">
         <v>2203</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O10" t="s">
         <v>2206</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>2166</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>2164</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>2152</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I11" t="s">
+        <v>2223</v>
+      </c>
+      <c r="J11" t="s">
         <v>2151</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K11" t="s">
         <v>2152</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M11" t="s">
         <v>2198</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N11" t="s">
         <v>2201</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O11" t="s">
         <v>2204</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>2167</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>2159</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>2160</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I12" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J12" t="s">
         <v>2161</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K12" t="s">
         <v>2160</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M12" t="s">
         <v>2200</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N12" t="s">
         <v>2203</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O12" t="s">
         <v>2206</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>2168</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>2169</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2152</v>
-      </c>
-      <c r="I12" t="s">
-        <v>2156</v>
-      </c>
-      <c r="J12" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L12" t="s">
-        <v>2199</v>
-      </c>
-      <c r="M12" t="s">
-        <v>2202</v>
-      </c>
-      <c r="N12" t="s">
-        <v>2205</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>2170</v>
-      </c>
-      <c r="B13" t="s">
-        <v>2155</v>
       </c>
       <c r="C13" t="s">
         <v>2152</v>
       </c>
       <c r="I13" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J13" t="s">
         <v>2156</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>2152</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>2199</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>2202</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>2205</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2152</v>
+      </c>
+      <c r="I14" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J14" t="s">
+        <v>2156</v>
+      </c>
+      <c r="K14" t="s">
+        <v>2152</v>
+      </c>
+      <c r="M14" t="s">
+        <v>2199</v>
+      </c>
+      <c r="N14" t="s">
+        <v>2202</v>
+      </c>
+      <c r="O14" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>2171</v>
-      </c>
-      <c r="B14" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>2173</v>
       </c>
       <c r="B15" t="s">
         <v>2172</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>2173</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>2174</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>2169</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>2152</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I17" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J17" t="s">
         <v>2156</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K17" t="s">
         <v>2152</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M17" t="s">
         <v>2199</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N17" t="s">
         <v>2202</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O17" t="s">
         <v>2205</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>2175</v>
-      </c>
-      <c r="B17" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>2176</v>
       </c>
       <c r="B18" t="s">
         <v>2172</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>2177</v>
+        <v>2176</v>
       </c>
       <c r="B19" t="s">
         <v>2172</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B20" t="s">
+        <v>2172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>2178</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>2179</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>2180</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2181</v>
-      </c>
-      <c r="C21" t="s">
-        <v>2160</v>
-      </c>
-      <c r="I21" t="s">
-        <v>2161</v>
-      </c>
-      <c r="J21" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L21" t="s">
-        <v>2200</v>
-      </c>
-      <c r="M21" t="s">
-        <v>2203</v>
-      </c>
-      <c r="N21" t="s">
-        <v>2206</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>2182</v>
       </c>
       <c r="B22" t="s">
         <v>2181</v>
@@ -7996,84 +8058,93 @@
         <v>2160</v>
       </c>
       <c r="I22" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J22" t="s">
         <v>2161</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>2160</v>
       </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>2200</v>
       </c>
-      <c r="M22" t="s">
+      <c r="N22" t="s">
         <v>2203</v>
       </c>
-      <c r="N22" t="s">
+      <c r="O22" t="s">
         <v>2206</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2181</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2160</v>
+      </c>
+      <c r="I23" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J23" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K23" t="s">
+        <v>2160</v>
+      </c>
+      <c r="M23" t="s">
+        <v>2200</v>
+      </c>
+      <c r="N23" t="s">
+        <v>2203</v>
+      </c>
+      <c r="O23" t="s">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>2183</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>2172</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>2184</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>2164</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" t="s">
         <v>2152</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I25" t="s">
+        <v>2223</v>
+      </c>
+      <c r="J25" t="s">
         <v>2151</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K25" t="s">
         <v>2152</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M25" t="s">
         <v>2198</v>
       </c>
-      <c r="M24" t="s">
+      <c r="N25" t="s">
         <v>2201</v>
       </c>
-      <c r="N24" t="s">
+      <c r="O25" t="s">
         <v>2204</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>2185</v>
-      </c>
-      <c r="B25" t="s">
-        <v>2186</v>
-      </c>
-      <c r="C25" t="s">
-        <v>2160</v>
-      </c>
-      <c r="I25" t="s">
-        <v>2161</v>
-      </c>
-      <c r="J25" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L25" t="s">
-        <v>2200</v>
-      </c>
-      <c r="M25" t="s">
-        <v>2203</v>
-      </c>
-      <c r="N25" t="s">
-        <v>2206</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>2187</v>
       </c>
       <c r="B26" t="s">
         <v>2186</v>
@@ -8081,30 +8152,62 @@
       <c r="C26" t="s">
         <v>2160</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I26" t="s">
+        <v>2225</v>
+      </c>
+      <c r="J26" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K26" t="s">
+        <v>2160</v>
+      </c>
+      <c r="M26" t="s">
+        <v>2200</v>
+      </c>
+      <c r="N26" t="s">
+        <v>2203</v>
+      </c>
+      <c r="O26" t="s">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>2187</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2186</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>2188</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>2169</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>2152</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I28" t="s">
+        <v>2224</v>
+      </c>
+      <c r="J28" t="s">
         <v>2156</v>
       </c>
-      <c r="J27" t="s">
+      <c r="K28" t="s">
         <v>2152</v>
       </c>
-      <c r="L27" t="s">
+      <c r="M28" t="s">
         <v>2199</v>
       </c>
-      <c r="M27" t="s">
+      <c r="N28" t="s">
         <v>2202</v>
       </c>
-      <c r="N27" t="s">
+      <c r="O28" t="s">
         <v>2205</v>
       </c>
     </row>
@@ -8308,10 +8411,10 @@
         <v>100</v>
       </c>
       <c r="C5" t="s">
+        <v>2219</v>
+      </c>
+      <c r="D5" t="s">
         <v>2220</v>
-      </c>
-      <c r="D5" t="s">
-        <v>2221</v>
       </c>
       <c r="E5" t="s">
         <v>101</v>
@@ -11787,7 +11890,7 @@
         <v>765</v>
       </c>
       <c r="C2" t="s">
-        <v>2218</v>
+        <v>2217</v>
       </c>
       <c r="D2" t="s">
         <v>766</v>
@@ -11869,28 +11972,28 @@
         <v>790</v>
       </c>
       <c r="C4" t="s">
+        <v>2210</v>
+      </c>
+      <c r="D4" t="s">
         <v>2211</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>2212</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>2213</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>2214</v>
-      </c>
-      <c r="G4" t="s">
-        <v>2215</v>
       </c>
       <c r="H4" t="s">
         <v>792</v>
       </c>
       <c r="I4" t="s">
-        <v>2217</v>
+        <v>2216</v>
       </c>
       <c r="J4" t="s">
-        <v>2216</v>
+        <v>2215</v>
       </c>
       <c r="K4" t="s">
         <v>793</v>
@@ -14907,7 +15010,7 @@
         <v>1467</v>
       </c>
       <c r="C59" t="s">
-        <v>2219</v>
+        <v>2218</v>
       </c>
       <c r="D59" t="s">
         <v>1468</v>

</xml_diff>

<commit_message>
cleaning out font cruft
</commit_message>
<xml_diff>
--- a/src/stp/database/localization.xlsx
+++ b/src/stp/database/localization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BF4CCB-7CCF-204E-8484-651459B61CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4CF6C1-1D0C-574C-9D6C-21A597656B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3571" uniqueCount="2261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3530" uniqueCount="2256">
   <si>
     <t>key</t>
   </si>
@@ -6481,15 +6481,9 @@
     <t>TradeGothicLTStd-LightObl.otf</t>
   </si>
   <si>
-    <t>calibrili.ttf</t>
-  </si>
-  <si>
     <t>YuGothL_0.ttf</t>
   </si>
   <si>
-    <t>calibri.ttf</t>
-  </si>
-  <si>
     <t>day.date</t>
   </si>
   <si>
@@ -6511,9 +6505,6 @@
     <t>TradeGothicLTStd-Bd2.otf</t>
   </si>
   <si>
-    <t>calibrib.ttf</t>
-  </si>
-  <si>
     <t>YuGothB_0.ttf</t>
   </si>
   <si>
@@ -6694,12 +6685,6 @@
     <t>Nordamerica</t>
   </si>
   <si>
-    <t>en_alt</t>
-  </si>
-  <si>
-    <t>ja_alt</t>
-  </si>
-  <si>
     <t>NotoSansCJKjp-Light.otf</t>
   </si>
   <si>
@@ -6745,9 +6730,6 @@
     <t>Name of Font files for each language. DO NOT CHANGE.</t>
   </si>
   <si>
-    <t>en_GB</t>
-  </si>
-  <si>
     <t>NotoSans-CondensedBold.otf</t>
   </si>
   <si>
@@ -6766,9 +6748,6 @@
     <t>NotoSans-Regular.otf</t>
   </si>
   <si>
-    <t>fa_af</t>
-  </si>
-  <si>
     <t>NotoSansArabic-ExtraBold.otf</t>
   </si>
   <si>
@@ -6812,6 +6791,12 @@
   </si>
   <si>
     <t>ماملودی سان‌داونز</t>
+  </si>
+  <si>
+    <t>en_orig</t>
+  </si>
+  <si>
+    <t>ja_orig</t>
   </si>
 </sst>
 </file>
@@ -6908,7 +6893,7 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6994,23 +6979,21 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}" name="Table10" displayName="Table10" ref="A2:L29" totalsRowShown="0">
-  <autoFilter ref="A2:L29" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:L29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}" name="Table10" displayName="Table10" ref="A2:J29" totalsRowShown="0">
+  <autoFilter ref="A2:J29" xr:uid="{C3230982-50AF-8C40-AE63-F916AAAD9846}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J29">
     <sortCondition ref="A2:A29"/>
   </sortState>
-  <tableColumns count="12">
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{ED366778-7374-0B4D-B3D7-3A1347569CE0}" name="key"/>
-    <tableColumn id="2" xr3:uid="{80E7518A-3634-0641-9EC4-DD7EB1B380BB}" name="en_GB"/>
-    <tableColumn id="3" xr3:uid="{FE7E56C3-4451-AE4D-B1AF-92EFC944B7F5}" name="en_alt"/>
+    <tableColumn id="2" xr3:uid="{80E7518A-3634-0641-9EC4-DD7EB1B380BB}" name="en_orig"/>
     <tableColumn id="16" xr3:uid="{220C42B2-F27C-5747-AEF1-1153C480D100}" name="en"/>
     <tableColumn id="15" xr3:uid="{B1CB1C0C-D5DA-524B-BC41-F9230EA4F8AA}" name="ja"/>
-    <tableColumn id="9" xr3:uid="{438BCE97-8A7A-EC4A-B263-6ECA8C0D3BB1}" name="ja_alt"/>
+    <tableColumn id="9" xr3:uid="{438BCE97-8A7A-EC4A-B263-6ECA8C0D3BB1}" name="ja_orig"/>
     <tableColumn id="12" xr3:uid="{AF687974-098A-8941-875B-EAFF0D8C9E19}" name="ko"/>
     <tableColumn id="13" xr3:uid="{9F259FFB-42AE-7C47-BDF2-C19F03F3E836}" name="zh_Hans"/>
     <tableColumn id="14" xr3:uid="{C7C15F4E-0CC4-8441-BFDF-C2D96356CF81}" name="zh_Hant"/>
     <tableColumn id="17" xr3:uid="{81818951-1E44-ED4D-8D2E-F3C9A51BF9E2}" name="fa" dataDxfId="0"/>
-    <tableColumn id="10" xr3:uid="{EAF98D58-A095-9C4F-918D-34BD7D07524B}" name="fa_af"/>
     <tableColumn id="18" xr3:uid="{F99DC2E5-03BC-1943-AC52-2AC76CA74AC6}" name="ar"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -7524,10 +7507,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2228</v>
+        <v>2223</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -7576,22 +7559,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -7795,27 +7778,25 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2237</v>
+        <v>2232</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -7825,48 +7806,40 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>2238</v>
+        <v>2254</v>
       </c>
       <c r="C2" t="s">
-        <v>2221</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>2255</v>
       </c>
       <c r="F2" t="s">
-        <v>2222</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>2205</v>
       </c>
       <c r="H2" t="s">
-        <v>2208</v>
+        <v>2206</v>
       </c>
       <c r="I2" t="s">
-        <v>2209</v>
+        <v>8</v>
       </c>
       <c r="J2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" t="s">
-        <v>2245</v>
-      </c>
-      <c r="L2" t="s">
-        <v>2257</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2148</v>
       </c>
@@ -7874,16 +7847,16 @@
         <v>2149</v>
       </c>
       <c r="C3" t="s">
+        <v>2237</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E3" t="s">
         <v>2150</v>
       </c>
-      <c r="D3" t="s">
-        <v>2243</v>
-      </c>
-      <c r="E3" t="s">
-        <v>2223</v>
-      </c>
       <c r="F3" t="s">
-        <v>2151</v>
+        <v>2195</v>
       </c>
       <c r="G3" t="s">
         <v>2198</v>
@@ -7892,74 +7865,62 @@
         <v>2201</v>
       </c>
       <c r="I3" t="s">
-        <v>2204</v>
+        <v>2243</v>
       </c>
       <c r="J3" t="s">
-        <v>2250</v>
-      </c>
-      <c r="K3" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L3" t="s">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2226</v>
+        <v>2221</v>
       </c>
       <c r="B4" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
       <c r="C4" t="s">
-        <v>2160</v>
+        <v>2234</v>
       </c>
       <c r="D4" t="s">
-        <v>2240</v>
+        <v>2245</v>
       </c>
       <c r="E4" t="s">
-        <v>2252</v>
+        <v>2158</v>
       </c>
       <c r="F4" t="s">
-        <v>2161</v>
+        <v>2246</v>
       </c>
       <c r="G4" t="s">
-        <v>2253</v>
+        <v>2247</v>
       </c>
       <c r="H4" t="s">
-        <v>2254</v>
+        <v>2248</v>
       </c>
       <c r="I4" t="s">
-        <v>2255</v>
+        <v>2239</v>
       </c>
       <c r="J4" t="s">
-        <v>2246</v>
-      </c>
-      <c r="K4" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L4" t="s">
-        <v>2246</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>2153</v>
+        <v>2151</v>
       </c>
       <c r="B5" t="s">
         <v>2149</v>
       </c>
       <c r="C5" t="s">
+        <v>2237</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E5" t="s">
         <v>2150</v>
       </c>
-      <c r="D5" t="s">
-        <v>2243</v>
-      </c>
-      <c r="E5" t="s">
-        <v>2223</v>
-      </c>
       <c r="F5" t="s">
-        <v>2151</v>
+        <v>2195</v>
       </c>
       <c r="G5" t="s">
         <v>2198</v>
@@ -7968,36 +7929,30 @@
         <v>2201</v>
       </c>
       <c r="I5" t="s">
-        <v>2204</v>
+        <v>2243</v>
       </c>
       <c r="J5" t="s">
-        <v>2250</v>
-      </c>
-      <c r="K5" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>2152</v>
       </c>
-      <c r="L5" t="s">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>2153</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2219</v>
+      </c>
+      <c r="E6" t="s">
         <v>2154</v>
       </c>
-      <c r="B6" t="s">
-        <v>2155</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>2244</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2224</v>
-      </c>
       <c r="F6" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G6" t="s">
         <v>2199</v>
@@ -8005,37 +7960,31 @@
       <c r="H6" t="s">
         <v>2202</v>
       </c>
-      <c r="I6" t="s">
-        <v>2205</v>
+      <c r="I6" s="5" t="s">
+        <v>2244</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>2251</v>
-      </c>
-      <c r="K6" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>2251</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>2157</v>
+        <v>2155</v>
       </c>
       <c r="B7" t="s">
-        <v>2155</v>
-      </c>
-      <c r="C7" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>2244</v>
+        <v>2153</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2219</v>
       </c>
       <c r="E7" t="s">
-        <v>2224</v>
+        <v>2154</v>
       </c>
       <c r="F7" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G7" t="s">
         <v>2199</v>
@@ -8043,113 +7992,95 @@
       <c r="H7" t="s">
         <v>2202</v>
       </c>
-      <c r="I7" t="s">
-        <v>2205</v>
+      <c r="I7" s="5" t="s">
+        <v>2244</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>2251</v>
-      </c>
-      <c r="K7" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>2251</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>2156</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2234</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2245</v>
+      </c>
+      <c r="E8" t="s">
         <v>2158</v>
       </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
+        <v>2246</v>
+      </c>
+      <c r="G8" t="s">
+        <v>2247</v>
+      </c>
+      <c r="H8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="I8" t="s">
+        <v>2239</v>
+      </c>
+      <c r="J8" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>2159</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B9" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2234</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2245</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F9" t="s">
+        <v>2246</v>
+      </c>
+      <c r="G9" t="s">
+        <v>2247</v>
+      </c>
+      <c r="H9" t="s">
+        <v>2248</v>
+      </c>
+      <c r="I9" t="s">
+        <v>2239</v>
+      </c>
+      <c r="J9" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>2160</v>
       </c>
-      <c r="D8" t="s">
-        <v>2240</v>
-      </c>
-      <c r="E8" t="s">
-        <v>2252</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="B10" t="s">
         <v>2161</v>
       </c>
-      <c r="G8" t="s">
-        <v>2253</v>
-      </c>
-      <c r="H8" t="s">
-        <v>2254</v>
-      </c>
-      <c r="I8" t="s">
-        <v>2255</v>
-      </c>
-      <c r="J8" t="s">
-        <v>2246</v>
-      </c>
-      <c r="K8" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L8" t="s">
-        <v>2246</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>2162</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2159</v>
-      </c>
-      <c r="C9" t="s">
-        <v>2160</v>
-      </c>
-      <c r="D9" t="s">
-        <v>2240</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2252</v>
-      </c>
-      <c r="F9" t="s">
-        <v>2161</v>
-      </c>
-      <c r="G9" t="s">
-        <v>2253</v>
-      </c>
-      <c r="H9" t="s">
-        <v>2254</v>
-      </c>
-      <c r="I9" t="s">
-        <v>2255</v>
-      </c>
-      <c r="J9" t="s">
-        <v>2246</v>
-      </c>
-      <c r="K9" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L9" t="s">
-        <v>2246</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>2163</v>
-      </c>
-      <c r="B10" t="s">
-        <v>2164</v>
-      </c>
       <c r="C10" t="s">
-        <v>2152</v>
+        <v>2236</v>
       </c>
       <c r="D10" t="s">
-        <v>2242</v>
+        <v>2218</v>
       </c>
       <c r="E10" t="s">
-        <v>2223</v>
+        <v>2150</v>
       </c>
       <c r="F10" t="s">
-        <v>2151</v>
+        <v>2195</v>
       </c>
       <c r="G10" t="s">
         <v>2198</v>
@@ -8158,74 +8089,62 @@
         <v>2201</v>
       </c>
       <c r="I10" t="s">
-        <v>2204</v>
+        <v>2243</v>
       </c>
       <c r="J10" t="s">
-        <v>2250</v>
-      </c>
-      <c r="K10" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L10" t="s">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>2165</v>
+        <v>2162</v>
       </c>
       <c r="B11" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
       <c r="C11" t="s">
-        <v>2160</v>
+        <v>2234</v>
       </c>
       <c r="D11" t="s">
-        <v>2240</v>
+        <v>2245</v>
       </c>
       <c r="E11" t="s">
-        <v>2252</v>
+        <v>2158</v>
       </c>
       <c r="F11" t="s">
+        <v>2246</v>
+      </c>
+      <c r="G11" t="s">
+        <v>2247</v>
+      </c>
+      <c r="H11" t="s">
+        <v>2248</v>
+      </c>
+      <c r="I11" t="s">
+        <v>2239</v>
+      </c>
+      <c r="J11" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>2163</v>
+      </c>
+      <c r="B12" t="s">
         <v>2161</v>
       </c>
-      <c r="G11" t="s">
-        <v>2253</v>
-      </c>
-      <c r="H11" t="s">
-        <v>2254</v>
-      </c>
-      <c r="I11" t="s">
-        <v>2255</v>
-      </c>
-      <c r="J11" t="s">
-        <v>2246</v>
-      </c>
-      <c r="K11" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L11" t="s">
-        <v>2246</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>2166</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2164</v>
-      </c>
       <c r="C12" t="s">
-        <v>2152</v>
+        <v>2236</v>
       </c>
       <c r="D12" t="s">
-        <v>2242</v>
+        <v>2218</v>
       </c>
       <c r="E12" t="s">
-        <v>2223</v>
+        <v>2150</v>
       </c>
       <c r="F12" t="s">
-        <v>2151</v>
+        <v>2195</v>
       </c>
       <c r="G12" t="s">
         <v>2198</v>
@@ -8234,74 +8153,62 @@
         <v>2201</v>
       </c>
       <c r="I12" t="s">
-        <v>2204</v>
+        <v>2243</v>
       </c>
       <c r="J12" t="s">
-        <v>2250</v>
-      </c>
-      <c r="K12" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L12" t="s">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>2167</v>
+        <v>2164</v>
       </c>
       <c r="B13" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
       <c r="C13" t="s">
-        <v>2160</v>
+        <v>2234</v>
       </c>
       <c r="D13" t="s">
-        <v>2240</v>
+        <v>2245</v>
       </c>
       <c r="E13" t="s">
-        <v>2252</v>
+        <v>2158</v>
       </c>
       <c r="F13" t="s">
-        <v>2161</v>
+        <v>2246</v>
       </c>
       <c r="G13" t="s">
-        <v>2253</v>
+        <v>2247</v>
       </c>
       <c r="H13" t="s">
-        <v>2254</v>
+        <v>2248</v>
       </c>
       <c r="I13" t="s">
-        <v>2255</v>
+        <v>2239</v>
       </c>
       <c r="J13" t="s">
-        <v>2246</v>
-      </c>
-      <c r="K13" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L13" t="s">
-        <v>2246</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>2168</v>
+        <v>2165</v>
       </c>
       <c r="B14" t="s">
-        <v>2169</v>
+        <v>2166</v>
       </c>
       <c r="C14" t="s">
-        <v>2152</v>
+        <v>2235</v>
       </c>
       <c r="D14" t="s">
-        <v>2241</v>
+        <v>2219</v>
       </c>
       <c r="E14" t="s">
-        <v>2224</v>
+        <v>2154</v>
       </c>
       <c r="F14" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G14" t="s">
         <v>2199</v>
@@ -8310,36 +8217,30 @@
         <v>2202</v>
       </c>
       <c r="I14" t="s">
-        <v>2205</v>
+        <v>2242</v>
       </c>
       <c r="J14" t="s">
-        <v>2249</v>
-      </c>
-      <c r="K14" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L14" t="s">
-        <v>2249</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>2170</v>
+        <v>2167</v>
       </c>
       <c r="B15" t="s">
-        <v>2155</v>
-      </c>
-      <c r="C15" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>2244</v>
+        <v>2153</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2219</v>
       </c>
       <c r="E15" t="s">
-        <v>2224</v>
+        <v>2154</v>
       </c>
       <c r="F15" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G15" t="s">
         <v>2199</v>
@@ -8347,59 +8248,53 @@
       <c r="H15" t="s">
         <v>2202</v>
       </c>
-      <c r="I15" t="s">
-        <v>2205</v>
+      <c r="I15" s="5" t="s">
+        <v>2244</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>2251</v>
-      </c>
-      <c r="K15" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>2251</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>2171</v>
       </c>
-      <c r="B16" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D16" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>2173</v>
-      </c>
-      <c r="B17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D17" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>2174</v>
-      </c>
       <c r="B18" t="s">
-        <v>2169</v>
+        <v>2166</v>
       </c>
       <c r="C18" t="s">
-        <v>2152</v>
+        <v>2235</v>
       </c>
       <c r="D18" t="s">
-        <v>2241</v>
+        <v>2219</v>
       </c>
       <c r="E18" t="s">
-        <v>2224</v>
+        <v>2154</v>
       </c>
       <c r="F18" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G18" t="s">
         <v>2199</v>
@@ -8408,80 +8303,74 @@
         <v>2202</v>
       </c>
       <c r="I18" t="s">
-        <v>2205</v>
+        <v>2242</v>
       </c>
       <c r="J18" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>2172</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>2173</v>
+      </c>
+      <c r="B20" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>2175</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2176</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2178</v>
+      </c>
+      <c r="C23" t="s">
         <v>2249</v>
       </c>
-      <c r="K18" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L18" t="s">
-        <v>2249</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>2175</v>
-      </c>
-      <c r="B19" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D19" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>2176</v>
-      </c>
-      <c r="B20" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D20" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>2177</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D21" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>2178</v>
-      </c>
-      <c r="B22" t="s">
-        <v>2179</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2179</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>2180</v>
-      </c>
-      <c r="B23" t="s">
-        <v>2181</v>
-      </c>
-      <c r="C23" t="s">
-        <v>2160</v>
-      </c>
       <c r="D23" t="s">
-        <v>2256</v>
+        <v>2220</v>
       </c>
       <c r="E23" t="s">
-        <v>2225</v>
+        <v>2158</v>
       </c>
       <c r="F23" t="s">
-        <v>2161</v>
+        <v>2197</v>
       </c>
       <c r="G23" t="s">
         <v>2200</v>
@@ -8490,36 +8379,30 @@
         <v>2203</v>
       </c>
       <c r="I23" t="s">
-        <v>2206</v>
+        <v>2241</v>
       </c>
       <c r="J23" t="s">
-        <v>2248</v>
-      </c>
-      <c r="K23" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L23" t="s">
-        <v>2248</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>2182</v>
+        <v>2179</v>
       </c>
       <c r="B24" t="s">
-        <v>2181</v>
+        <v>2178</v>
       </c>
       <c r="C24" t="s">
-        <v>2160</v>
+        <v>2249</v>
       </c>
       <c r="D24" t="s">
-        <v>2256</v>
+        <v>2220</v>
       </c>
       <c r="E24" t="s">
-        <v>2225</v>
+        <v>2158</v>
       </c>
       <c r="F24" t="s">
-        <v>2161</v>
+        <v>2197</v>
       </c>
       <c r="G24" t="s">
         <v>2200</v>
@@ -8528,47 +8411,41 @@
         <v>2203</v>
       </c>
       <c r="I24" t="s">
-        <v>2206</v>
+        <v>2241</v>
       </c>
       <c r="J24" t="s">
-        <v>2248</v>
-      </c>
-      <c r="K24" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L24" t="s">
-        <v>2248</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>2183</v>
+        <v>2180</v>
       </c>
       <c r="B25" t="s">
-        <v>2172</v>
-      </c>
-      <c r="D25" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2169</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>2184</v>
+        <v>2181</v>
       </c>
       <c r="B26" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
       <c r="C26" t="s">
-        <v>2152</v>
+        <v>2236</v>
       </c>
       <c r="D26" t="s">
-        <v>2242</v>
+        <v>2218</v>
       </c>
       <c r="E26" t="s">
-        <v>2223</v>
+        <v>2150</v>
       </c>
       <c r="F26" t="s">
-        <v>2151</v>
+        <v>2195</v>
       </c>
       <c r="G26" t="s">
         <v>2198</v>
@@ -8577,52 +8454,43 @@
         <v>2201</v>
       </c>
       <c r="I26" t="s">
-        <v>2204</v>
+        <v>2243</v>
       </c>
       <c r="J26" t="s">
-        <v>2250</v>
-      </c>
-      <c r="K26" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L26" t="s">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>2187</v>
+        <v>2184</v>
       </c>
       <c r="B27" t="s">
-        <v>2186</v>
-      </c>
-      <c r="C27" t="s">
-        <v>2160</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>2239</v>
-      </c>
+        <v>2183</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>2233</v>
+      </c>
+      <c r="I27" s="6"/>
       <c r="J27" s="6"/>
-      <c r="L27" s="6"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>2185</v>
+        <v>2182</v>
       </c>
       <c r="B28" t="s">
-        <v>2186</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2160</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>2239</v>
+        <v>2183</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>2233</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2220</v>
       </c>
       <c r="E28" t="s">
-        <v>2225</v>
+        <v>2158</v>
       </c>
       <c r="F28" t="s">
-        <v>2161</v>
+        <v>2197</v>
       </c>
       <c r="G28" t="s">
         <v>2200</v>
@@ -8630,37 +8498,31 @@
       <c r="H28" t="s">
         <v>2203</v>
       </c>
-      <c r="I28" t="s">
-        <v>2206</v>
+      <c r="I28" s="6" t="s">
+        <v>2240</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>2247</v>
-      </c>
-      <c r="K28" t="s">
-        <v>2160</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>2247</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>2188</v>
+        <v>2185</v>
       </c>
       <c r="B29" t="s">
-        <v>2169</v>
-      </c>
-      <c r="C29" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>2241</v>
+        <v>2166</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D29" t="s">
+        <v>2219</v>
       </c>
       <c r="E29" t="s">
-        <v>2224</v>
+        <v>2154</v>
       </c>
       <c r="F29" t="s">
-        <v>2156</v>
+        <v>2196</v>
       </c>
       <c r="G29" t="s">
         <v>2199</v>
@@ -8668,17 +8530,11 @@
       <c r="H29" t="s">
         <v>2202</v>
       </c>
-      <c r="I29" t="s">
-        <v>2205</v>
+      <c r="I29" s="6" t="s">
+        <v>2242</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>2249</v>
-      </c>
-      <c r="K29" t="s">
-        <v>2152</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>2249</v>
+        <v>2242</v>
       </c>
     </row>
   </sheetData>
@@ -8712,10 +8568,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2229</v>
+        <v>2224</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -8764,22 +8620,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -8913,10 +8769,10 @@
         <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>2219</v>
+        <v>2216</v>
       </c>
       <c r="D6" t="s">
-        <v>2220</v>
+        <v>2217</v>
       </c>
       <c r="E6" t="s">
         <v>101</v>
@@ -9182,10 +9038,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2230</v>
+        <v>2225</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -9234,22 +9090,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -10347,7 +10203,7 @@
         <v>376</v>
       </c>
       <c r="J29" t="s">
-        <v>2207</v>
+        <v>2204</v>
       </c>
       <c r="K29" t="s">
         <v>379</v>
@@ -12147,10 +12003,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2231</v>
+        <v>2226</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -12199,22 +12055,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -12414,10 +12270,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>2222</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>2227</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2232</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -12466,22 +12322,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -12492,7 +12348,7 @@
         <v>765</v>
       </c>
       <c r="C3" t="s">
-        <v>2217</v>
+        <v>2214</v>
       </c>
       <c r="D3" t="s">
         <v>766</v>
@@ -12574,22 +12430,22 @@
         <v>790</v>
       </c>
       <c r="C5" t="s">
+        <v>2207</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2208</v>
+      </c>
+      <c r="E5" t="s">
+        <v>2209</v>
+      </c>
+      <c r="F5" t="s">
         <v>2210</v>
       </c>
-      <c r="D5" t="s">
+      <c r="G5" t="s">
         <v>2211</v>
       </c>
-      <c r="E5" t="s">
+      <c r="H5" t="s">
         <v>2212</v>
-      </c>
-      <c r="F5" t="s">
-        <v>2213</v>
-      </c>
-      <c r="G5" t="s">
-        <v>2214</v>
-      </c>
-      <c r="H5" t="s">
-        <v>2215</v>
       </c>
       <c r="I5" t="s">
         <v>792</v>
@@ -12604,7 +12460,7 @@
         <v>795</v>
       </c>
       <c r="M5" t="s">
-        <v>2216</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -12630,7 +12486,7 @@
         <v>801</v>
       </c>
       <c r="H6" t="s">
-        <v>2189</v>
+        <v>2186</v>
       </c>
       <c r="I6" t="s">
         <v>802</v>
@@ -12671,7 +12527,7 @@
         <v>813</v>
       </c>
       <c r="H7" t="s">
-        <v>2190</v>
+        <v>2187</v>
       </c>
       <c r="I7" t="s">
         <v>814</v>
@@ -12842,10 +12698,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2233</v>
+        <v>2228</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -12894,22 +12750,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -13008,13 +12864,13 @@
         <v>877</v>
       </c>
       <c r="E5" t="s">
+        <v>2188</v>
+      </c>
+      <c r="F5" t="s">
         <v>2191</v>
       </c>
-      <c r="F5" t="s">
-        <v>2194</v>
-      </c>
       <c r="G5" t="s">
-        <v>2195</v>
+        <v>2192</v>
       </c>
       <c r="H5" t="s">
         <v>880</v>
@@ -13043,22 +12899,22 @@
         <v>885</v>
       </c>
       <c r="C6" t="s">
-        <v>2193</v>
+        <v>2190</v>
       </c>
       <c r="D6" t="s">
         <v>888</v>
       </c>
       <c r="E6" t="s">
-        <v>2192</v>
+        <v>2189</v>
       </c>
       <c r="F6" t="s">
-        <v>2197</v>
+        <v>2194</v>
       </c>
       <c r="G6" t="s">
-        <v>2196</v>
+        <v>2193</v>
       </c>
       <c r="H6" t="s">
-        <v>2193</v>
+        <v>2190</v>
       </c>
       <c r="I6" t="s">
         <v>886</v>
@@ -13107,10 +12963,10 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2234</v>
+        <v>2229</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -13163,22 +13019,22 @@
         <v>10</v>
       </c>
       <c r="L2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="M2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="N2" t="s">
         <v>8</v>
       </c>
       <c r="O2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="P2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="Q2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -13300,10 +13156,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2235</v>
+        <v>2230</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -13352,22 +13208,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -15715,7 +15571,7 @@
         <v>1467</v>
       </c>
       <c r="C60" t="s">
-        <v>2218</v>
+        <v>2215</v>
       </c>
       <c r="D60" t="s">
         <v>1468</v>
@@ -17463,10 +17319,10 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2236</v>
+        <v>2231</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -17515,22 +17371,22 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>2208</v>
+        <v>2205</v>
       </c>
       <c r="L2" t="s">
-        <v>2209</v>
+        <v>2206</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>2257</v>
+        <v>2250</v>
       </c>
       <c r="O2" t="s">
-        <v>2258</v>
+        <v>2251</v>
       </c>
       <c r="P2" t="s">
-        <v>2259</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -18514,7 +18370,7 @@
         <v>2072</v>
       </c>
       <c r="M26" t="s">
-        <v>2260</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
venues - turkish text and russian corrections
</commit_message>
<xml_diff>
--- a/src/stp/database/localization.xlsx
+++ b/src/stp/database/localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B6E0A1-8EB6-8342-BBB1-2EEEF45E3882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF29C63-279E-9E46-B3D5-FE0F306AA645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Competition" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4186" uniqueCount="2790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4256" uniqueCount="2809">
   <si>
     <t>key</t>
   </si>
@@ -7003,15 +7003,9 @@
     <t>«Аль-Байт»</t>
   </si>
   <si>
-    <t> «Аль-Джануб»</t>
-  </si>
-  <si>
     <t>«Аль-Тумама»</t>
   </si>
   <si>
-    <t> «Эдьюкейшн сити»</t>
-  </si>
-  <si>
     <t>«Халифа Интернейшнл»</t>
   </si>
   <si>
@@ -7057,75 +7051,6 @@
     <t>Волгоград</t>
   </si>
   <si>
-    <t>Арлингтон, Техас</t>
-  </si>
-  <si>
-    <t>Атланта, Джорджия</t>
-  </si>
-  <si>
-    <t>Остин, Техас</t>
-  </si>
-  <si>
-    <t>Бостон, Массачусетс</t>
-  </si>
-  <si>
-    <t>Шарлотт, Сев. Каролина</t>
-  </si>
-  <si>
-    <t> Цинциннати, Огайо</t>
-  </si>
-  <si>
-    <t>Даллас, Техас</t>
-  </si>
-  <si>
-    <t>Ист-Ратерфорд, Нью-Джерси</t>
-  </si>
-  <si>
-    <t>Глендейл, Аризона</t>
-  </si>
-  <si>
-    <t>Хьюстон, Техас</t>
-  </si>
-  <si>
-    <t>Инглвуд, Калифорния</t>
-  </si>
-  <si>
-    <t> Канзас-Сити, Канзас</t>
-  </si>
-  <si>
-    <t>Канзас-Сити, Миссури</t>
-  </si>
-  <si>
-    <t>Лас-Вегас, Невада</t>
-  </si>
-  <si>
-    <t>Лос-Анджелес, Калифорния</t>
-  </si>
-  <si>
-    <t>Майами, Флорида</t>
-  </si>
-  <si>
-    <t>Нэшвилл, Теннеси</t>
-  </si>
-  <si>
-    <t>Орландо, Флорида</t>
-  </si>
-  <si>
-    <t>Пасадена, Калифорния</t>
-  </si>
-  <si>
-    <t>Филадельфия, Пенсильвания</t>
-  </si>
-  <si>
-    <t>Санта-Клара, Калифорния</t>
-  </si>
-  <si>
-    <t>Сиэтл, Вашингтон</t>
-  </si>
-  <si>
-    <t>Вашингтон, округ Колумбия</t>
-  </si>
-  <si>
     <t>أديلايد</t>
   </si>
   <si>
@@ -8399,6 +8324,138 @@
   </si>
   <si>
     <t>El-Hilâl</t>
+  </si>
+  <si>
+    <t>Sidney</t>
+  </si>
+  <si>
+    <t>Avustralya Stadyumu</t>
+  </si>
+  <si>
+    <t>Sidney Futbol Stadyumu</t>
+  </si>
+  <si>
+    <t>Münih</t>
+  </si>
+  <si>
+    <t>Meksiko</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stadyum 974 </t>
+  </si>
+  <si>
+    <t>Ahmed bin Ali</t>
+  </si>
+  <si>
+    <t>El-Beyt</t>
+  </si>
+  <si>
+    <t>El-Cenub</t>
+  </si>
+  <si>
+    <t>Es-Sümame</t>
+  </si>
+  <si>
+    <t>Eğitim Şehri</t>
+  </si>
+  <si>
+    <t>Uluslararası Halife Stadyumu</t>
+  </si>
+  <si>
+    <t>Luseyl</t>
+  </si>
+  <si>
+    <t>Yekaterinburg</t>
+  </si>
+  <si>
+    <t>Moskova</t>
+  </si>
+  <si>
+    <t>Lujniki Stadyumu</t>
+  </si>
+  <si>
+    <t>Otkrıtiye Arena</t>
+  </si>
+  <si>
+    <t>Rostov-na-Donu</t>
+  </si>
+  <si>
+    <t>Sankt-Peterburg</t>
+  </si>
+  <si>
+    <t>Soçi</t>
+  </si>
+  <si>
+    <t>Арлингтон</t>
+  </si>
+  <si>
+    <t>Атланта</t>
+  </si>
+  <si>
+    <t>Остин</t>
+  </si>
+  <si>
+    <t>Бостон</t>
+  </si>
+  <si>
+    <t>Шарлотт</t>
+  </si>
+  <si>
+    <t>Даллас</t>
+  </si>
+  <si>
+    <t>Ист-Ратерфорд</t>
+  </si>
+  <si>
+    <t>Глендейл</t>
+  </si>
+  <si>
+    <t>Хьюстон</t>
+  </si>
+  <si>
+    <t>Инглвуд</t>
+  </si>
+  <si>
+    <t>Канзас-Сити, MO</t>
+  </si>
+  <si>
+    <t>Лас-Вегас</t>
+  </si>
+  <si>
+    <t>Майами</t>
+  </si>
+  <si>
+    <t>Нэшвилл</t>
+  </si>
+  <si>
+    <t>Орландо</t>
+  </si>
+  <si>
+    <t>Пасадена</t>
+  </si>
+  <si>
+    <t>Филадельфия</t>
+  </si>
+  <si>
+    <t>Санта-Клара</t>
+  </si>
+  <si>
+    <t>Сиэтл</t>
+  </si>
+  <si>
+    <t>Вашингтон, DC</t>
+  </si>
+  <si>
+    <t>Цинциннати</t>
+  </si>
+  <si>
+    <t>Канзас-Сити, KS</t>
+  </si>
+  <si>
+    <t>«Аль-Джануб»</t>
+  </si>
+  <si>
+    <t>«Эдьюкейшн сити»</t>
   </si>
 </sst>
 </file>
@@ -10802,7 +10859,7 @@
     <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="28" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
@@ -10918,10 +10975,13 @@
         <v>168</v>
       </c>
       <c r="N3" t="s">
-        <v>2365</v>
+        <v>2340</v>
       </c>
       <c r="O3" t="s">
         <v>2295</v>
+      </c>
+      <c r="P3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -10965,10 +11025,13 @@
         <v>175</v>
       </c>
       <c r="N4" t="s">
-        <v>2366</v>
+        <v>2341</v>
       </c>
       <c r="O4" t="s">
         <v>2296</v>
+      </c>
+      <c r="P4" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -11017,6 +11080,9 @@
       <c r="O5" t="s">
         <v>2297</v>
       </c>
+      <c r="P5" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -11059,10 +11125,13 @@
         <v>189</v>
       </c>
       <c r="N6" t="s">
-        <v>2367</v>
+        <v>2342</v>
       </c>
       <c r="O6" t="s">
         <v>2298</v>
+      </c>
+      <c r="P6" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -11106,10 +11175,13 @@
         <v>196</v>
       </c>
       <c r="N7" t="s">
-        <v>2368</v>
+        <v>2343</v>
       </c>
       <c r="O7" t="s">
         <v>2299</v>
+      </c>
+      <c r="P7" t="s">
+        <v>2765</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -11153,10 +11225,13 @@
         <v>206</v>
       </c>
       <c r="N8" t="s">
-        <v>2369</v>
+        <v>2344</v>
       </c>
       <c r="O8" t="s">
         <v>2300</v>
+      </c>
+      <c r="P8" t="s">
+        <v>2766</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -11200,10 +11275,13 @@
         <v>215</v>
       </c>
       <c r="N9" t="s">
-        <v>2370</v>
+        <v>2345</v>
       </c>
       <c r="O9" t="s">
         <v>2301</v>
+      </c>
+      <c r="P9" t="s">
+        <v>2767</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -11247,10 +11325,13 @@
         <v>220</v>
       </c>
       <c r="N10" t="s">
-        <v>2371</v>
+        <v>2346</v>
       </c>
       <c r="O10" t="s">
         <v>2302</v>
+      </c>
+      <c r="P10" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -11294,10 +11375,13 @@
         <v>227</v>
       </c>
       <c r="N11" t="s">
-        <v>2372</v>
+        <v>2347</v>
       </c>
       <c r="O11" t="s">
         <v>2303</v>
+      </c>
+      <c r="P11" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -11341,10 +11425,13 @@
         <v>237</v>
       </c>
       <c r="N12" t="s">
-        <v>2373</v>
+        <v>2348</v>
       </c>
       <c r="O12" t="s">
         <v>2304</v>
+      </c>
+      <c r="P12" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -11388,10 +11475,13 @@
         <v>247</v>
       </c>
       <c r="N13" t="s">
-        <v>2374</v>
+        <v>2349</v>
       </c>
       <c r="O13" t="s">
         <v>2305</v>
+      </c>
+      <c r="P13" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -11440,6 +11530,9 @@
       <c r="O14" t="s">
         <v>2306</v>
       </c>
+      <c r="P14" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -11487,6 +11580,9 @@
       <c r="O15" t="s">
         <v>2307</v>
       </c>
+      <c r="P15" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -11529,13 +11625,16 @@
         <v>270</v>
       </c>
       <c r="N16" t="s">
-        <v>2375</v>
+        <v>2350</v>
       </c>
       <c r="O16" t="s">
         <v>2308</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P16" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>274</v>
       </c>
@@ -11576,13 +11675,16 @@
         <v>277</v>
       </c>
       <c r="N17" t="s">
-        <v>2376</v>
+        <v>2351</v>
       </c>
       <c r="O17" t="s">
         <v>2309</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P17" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>281</v>
       </c>
@@ -11623,13 +11725,16 @@
         <v>287</v>
       </c>
       <c r="N18" t="s">
-        <v>2377</v>
+        <v>2352</v>
       </c>
       <c r="O18" t="s">
         <v>2310</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P18" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>291</v>
       </c>
@@ -11670,13 +11775,16 @@
         <v>295</v>
       </c>
       <c r="N19" t="s">
-        <v>2378</v>
+        <v>2353</v>
       </c>
       <c r="O19" t="s">
         <v>2311</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P19" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>299</v>
       </c>
@@ -11717,13 +11825,16 @@
         <v>305</v>
       </c>
       <c r="N20" t="s">
-        <v>2379</v>
+        <v>2354</v>
       </c>
       <c r="O20" t="s">
         <v>2312</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P20" t="s">
+        <v>2768</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>309</v>
       </c>
@@ -11764,13 +11875,16 @@
         <v>313</v>
       </c>
       <c r="N21" t="s">
-        <v>2380</v>
+        <v>2355</v>
       </c>
       <c r="O21" t="s">
         <v>2313</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P21" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>317</v>
       </c>
@@ -11811,13 +11925,16 @@
         <v>320</v>
       </c>
       <c r="N22" t="s">
-        <v>2381</v>
+        <v>2356</v>
       </c>
       <c r="O22" t="s">
         <v>2314</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P22" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>324</v>
       </c>
@@ -11858,13 +11975,16 @@
         <v>332</v>
       </c>
       <c r="N23" t="s">
-        <v>2382</v>
+        <v>2357</v>
       </c>
       <c r="O23" t="s">
         <v>2315</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P23" t="s">
+        <v>2769</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>336</v>
       </c>
@@ -11905,13 +12025,16 @@
         <v>339</v>
       </c>
       <c r="N24" t="s">
-        <v>2383</v>
+        <v>2358</v>
       </c>
       <c r="O24" t="s">
         <v>2316</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P24" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>342</v>
       </c>
@@ -11952,13 +12075,16 @@
         <v>345</v>
       </c>
       <c r="N25" t="s">
-        <v>2384</v>
+        <v>2359</v>
       </c>
       <c r="O25" t="s">
         <v>2317</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P25" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>349</v>
       </c>
@@ -11999,13 +12125,16 @@
         <v>352</v>
       </c>
       <c r="N26" t="s">
-        <v>2385</v>
+        <v>2360</v>
       </c>
       <c r="O26" t="s">
         <v>2318</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P26" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>356</v>
       </c>
@@ -12046,13 +12175,16 @@
         <v>359</v>
       </c>
       <c r="N27" t="s">
-        <v>2386</v>
+        <v>2361</v>
       </c>
       <c r="O27" t="s">
         <v>2319</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P27" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>363</v>
       </c>
@@ -12093,13 +12225,16 @@
         <v>366</v>
       </c>
       <c r="N28" t="s">
-        <v>2387</v>
+        <v>2362</v>
       </c>
       <c r="O28" t="s">
         <v>2320</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P28" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>370</v>
       </c>
@@ -12140,13 +12275,16 @@
         <v>377</v>
       </c>
       <c r="N29" t="s">
-        <v>2388</v>
+        <v>2363</v>
       </c>
       <c r="O29" t="s">
         <v>2321</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P29" t="s">
+        <v>2770</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>381</v>
       </c>
@@ -12187,13 +12325,16 @@
         <v>384</v>
       </c>
       <c r="N30" t="s">
-        <v>2389</v>
+        <v>2364</v>
       </c>
       <c r="O30" t="s">
         <v>2322</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P30" t="s">
+        <v>2771</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>388</v>
       </c>
@@ -12239,8 +12380,11 @@
       <c r="O31" t="s">
         <v>2323</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P31" t="s">
+        <v>2772</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>394</v>
       </c>
@@ -12284,10 +12428,13 @@
         <v>397</v>
       </c>
       <c r="O32" t="s">
-        <v>2324</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2807</v>
+      </c>
+      <c r="P32" t="s">
+        <v>2773</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>401</v>
       </c>
@@ -12331,10 +12478,13 @@
         <v>404</v>
       </c>
       <c r="O33" t="s">
-        <v>2325</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2324</v>
+      </c>
+      <c r="P33" t="s">
+        <v>2774</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>408</v>
       </c>
@@ -12375,13 +12525,16 @@
         <v>411</v>
       </c>
       <c r="N34" t="s">
-        <v>2390</v>
+        <v>2365</v>
       </c>
       <c r="O34" t="s">
-        <v>2326</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2808</v>
+      </c>
+      <c r="P34" t="s">
+        <v>2775</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>414</v>
       </c>
@@ -12422,13 +12575,16 @@
         <v>417</v>
       </c>
       <c r="N35" t="s">
-        <v>2391</v>
+        <v>2366</v>
       </c>
       <c r="O35" t="s">
-        <v>2327</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2325</v>
+      </c>
+      <c r="P35" t="s">
+        <v>2776</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>422</v>
       </c>
@@ -12469,13 +12625,16 @@
         <v>425</v>
       </c>
       <c r="N36" t="s">
-        <v>2392</v>
+        <v>2367</v>
       </c>
       <c r="O36" t="s">
-        <v>2328</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2326</v>
+      </c>
+      <c r="P36" t="s">
+        <v>2777</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>429</v>
       </c>
@@ -12516,13 +12675,16 @@
         <v>436</v>
       </c>
       <c r="N37" t="s">
-        <v>2393</v>
+        <v>2368</v>
       </c>
       <c r="O37" t="s">
-        <v>2329</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2327</v>
+      </c>
+      <c r="P37" t="s">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>441</v>
       </c>
@@ -12563,13 +12725,16 @@
         <v>445</v>
       </c>
       <c r="N38" t="s">
-        <v>2394</v>
+        <v>2369</v>
       </c>
       <c r="O38" t="s">
-        <v>2330</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2328</v>
+      </c>
+      <c r="P38" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>449</v>
       </c>
@@ -12610,13 +12775,16 @@
         <v>454</v>
       </c>
       <c r="N39" t="s">
-        <v>2395</v>
+        <v>2370</v>
       </c>
       <c r="O39" t="s">
-        <v>2331</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2329</v>
+      </c>
+      <c r="P39" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>457</v>
       </c>
@@ -12657,13 +12825,16 @@
         <v>465</v>
       </c>
       <c r="N40" t="s">
-        <v>2396</v>
+        <v>2371</v>
       </c>
       <c r="O40" t="s">
-        <v>2332</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2330</v>
+      </c>
+      <c r="P40" t="s">
+        <v>2779</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>468</v>
       </c>
@@ -12704,13 +12875,16 @@
         <v>476</v>
       </c>
       <c r="N41" t="s">
-        <v>2397</v>
+        <v>2372</v>
       </c>
       <c r="O41" t="s">
-        <v>2333</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2331</v>
+      </c>
+      <c r="P41" t="s">
+        <v>2780</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>481</v>
       </c>
@@ -12751,13 +12925,16 @@
         <v>484</v>
       </c>
       <c r="N42" t="s">
-        <v>2398</v>
+        <v>2373</v>
       </c>
       <c r="O42" t="s">
-        <v>2334</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2332</v>
+      </c>
+      <c r="P42" t="s">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>489</v>
       </c>
@@ -12798,13 +12975,16 @@
         <v>497</v>
       </c>
       <c r="N43" t="s">
-        <v>2399</v>
+        <v>2374</v>
       </c>
       <c r="O43" t="s">
-        <v>2335</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2333</v>
+      </c>
+      <c r="P43" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>501</v>
       </c>
@@ -12845,13 +13025,16 @@
         <v>509</v>
       </c>
       <c r="N44" t="s">
-        <v>2400</v>
+        <v>2375</v>
       </c>
       <c r="O44" t="s">
-        <v>2336</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2334</v>
+      </c>
+      <c r="P44" t="s">
+        <v>2782</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>513</v>
       </c>
@@ -12892,13 +13075,16 @@
         <v>521</v>
       </c>
       <c r="N45" t="s">
-        <v>2401</v>
+        <v>2376</v>
       </c>
       <c r="O45" t="s">
-        <v>2337</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2335</v>
+      </c>
+      <c r="P45" t="s">
+        <v>2783</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>526</v>
       </c>
@@ -12942,10 +13128,13 @@
         <v>529</v>
       </c>
       <c r="O46" t="s">
-        <v>2338</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2336</v>
+      </c>
+      <c r="P46" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>533</v>
       </c>
@@ -12986,13 +13175,16 @@
         <v>536</v>
       </c>
       <c r="N47" t="s">
-        <v>2402</v>
+        <v>2377</v>
       </c>
       <c r="O47" t="s">
-        <v>2339</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2337</v>
+      </c>
+      <c r="P47" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>540</v>
       </c>
@@ -13033,13 +13225,16 @@
         <v>547</v>
       </c>
       <c r="N48" t="s">
-        <v>2403</v>
+        <v>2378</v>
       </c>
       <c r="O48" t="s">
-        <v>2340</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2338</v>
+      </c>
+      <c r="P48" t="s">
+        <v>2784</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>550</v>
       </c>
@@ -13080,13 +13275,16 @@
         <v>555</v>
       </c>
       <c r="N49" t="s">
-        <v>2404</v>
+        <v>2379</v>
       </c>
       <c r="O49" t="s">
-        <v>2341</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2339</v>
+      </c>
+      <c r="P49" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>559</v>
       </c>
@@ -13127,13 +13325,16 @@
         <v>562</v>
       </c>
       <c r="N50" t="s">
-        <v>2405</v>
+        <v>2380</v>
       </c>
       <c r="O50" t="s">
-        <v>2342</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2785</v>
+      </c>
+      <c r="P50" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>566</v>
       </c>
@@ -13174,13 +13375,16 @@
         <v>569</v>
       </c>
       <c r="N51" t="s">
-        <v>2406</v>
+        <v>2381</v>
       </c>
       <c r="O51" t="s">
-        <v>2343</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2786</v>
+      </c>
+      <c r="P51" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>573</v>
       </c>
@@ -13221,13 +13425,16 @@
         <v>576</v>
       </c>
       <c r="N52" t="s">
-        <v>2407</v>
+        <v>2382</v>
       </c>
       <c r="O52" t="s">
-        <v>2344</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2787</v>
+      </c>
+      <c r="P52" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>580</v>
       </c>
@@ -13268,13 +13475,16 @@
         <v>583</v>
       </c>
       <c r="N53" t="s">
-        <v>2408</v>
+        <v>2383</v>
       </c>
       <c r="O53" t="s">
-        <v>2345</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2788</v>
+      </c>
+      <c r="P53" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>587</v>
       </c>
@@ -13318,10 +13528,13 @@
         <v>590</v>
       </c>
       <c r="O54" t="s">
-        <v>2346</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2789</v>
+      </c>
+      <c r="P54" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>593</v>
       </c>
@@ -13362,13 +13575,16 @@
         <v>596</v>
       </c>
       <c r="N55" t="s">
-        <v>2409</v>
+        <v>2384</v>
       </c>
       <c r="O55" t="s">
-        <v>2347</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2805</v>
+      </c>
+      <c r="P55" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>599</v>
       </c>
@@ -13412,10 +13628,13 @@
         <v>602</v>
       </c>
       <c r="O56" t="s">
-        <v>2348</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2790</v>
+      </c>
+      <c r="P56" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>606</v>
       </c>
@@ -13456,13 +13675,16 @@
         <v>609</v>
       </c>
       <c r="N57" t="s">
-        <v>2410</v>
+        <v>2385</v>
       </c>
       <c r="O57" t="s">
-        <v>2349</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2791</v>
+      </c>
+      <c r="P57" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>613</v>
       </c>
@@ -13503,13 +13725,16 @@
         <v>616</v>
       </c>
       <c r="N58" t="s">
-        <v>2411</v>
+        <v>2386</v>
       </c>
       <c r="O58" t="s">
-        <v>2350</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2792</v>
+      </c>
+      <c r="P58" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>620</v>
       </c>
@@ -13550,13 +13775,16 @@
         <v>623</v>
       </c>
       <c r="N59" t="s">
-        <v>2412</v>
+        <v>2387</v>
       </c>
       <c r="O59" t="s">
-        <v>2351</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2793</v>
+      </c>
+      <c r="P59" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>626</v>
       </c>
@@ -13597,13 +13825,16 @@
         <v>629</v>
       </c>
       <c r="N60" t="s">
-        <v>2413</v>
+        <v>2388</v>
       </c>
       <c r="O60" t="s">
-        <v>2352</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2794</v>
+      </c>
+      <c r="P60" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>633</v>
       </c>
@@ -13644,13 +13875,16 @@
         <v>636</v>
       </c>
       <c r="N61" t="s">
-        <v>2414</v>
+        <v>2389</v>
       </c>
       <c r="O61" t="s">
-        <v>2353</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2806</v>
+      </c>
+      <c r="P61" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>640</v>
       </c>
@@ -13691,13 +13925,16 @@
         <v>643</v>
       </c>
       <c r="N62" t="s">
-        <v>2415</v>
+        <v>2390</v>
       </c>
       <c r="O62" t="s">
-        <v>2354</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2795</v>
+      </c>
+      <c r="P62" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>647</v>
       </c>
@@ -13738,13 +13975,16 @@
         <v>650</v>
       </c>
       <c r="N63" t="s">
-        <v>2416</v>
+        <v>2391</v>
       </c>
       <c r="O63" t="s">
-        <v>2355</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2796</v>
+      </c>
+      <c r="P63" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>654</v>
       </c>
@@ -13785,13 +14025,16 @@
         <v>658</v>
       </c>
       <c r="N64" t="s">
-        <v>2417</v>
+        <v>2392</v>
       </c>
       <c r="O64" t="s">
-        <v>2356</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2759</v>
+      </c>
+      <c r="P64" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>662</v>
       </c>
@@ -13832,13 +14075,16 @@
         <v>665</v>
       </c>
       <c r="N65" t="s">
-        <v>2418</v>
+        <v>2393</v>
       </c>
       <c r="O65" t="s">
-        <v>2357</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2797</v>
+      </c>
+      <c r="P65" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>669</v>
       </c>
@@ -13879,13 +14125,16 @@
         <v>672</v>
       </c>
       <c r="N66" t="s">
-        <v>2419</v>
+        <v>2394</v>
       </c>
       <c r="O66" t="s">
-        <v>2358</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2798</v>
+      </c>
+      <c r="P66" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>676</v>
       </c>
@@ -13926,13 +14175,16 @@
         <v>679</v>
       </c>
       <c r="N67" t="s">
-        <v>2420</v>
+        <v>2395</v>
       </c>
       <c r="O67" t="s">
-        <v>2359</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2799</v>
+      </c>
+      <c r="P67" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>683</v>
       </c>
@@ -13973,13 +14225,16 @@
         <v>686</v>
       </c>
       <c r="N68" t="s">
-        <v>2421</v>
+        <v>2396</v>
       </c>
       <c r="O68" t="s">
-        <v>2360</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2800</v>
+      </c>
+      <c r="P68" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>690</v>
       </c>
@@ -14020,13 +14275,16 @@
         <v>693</v>
       </c>
       <c r="N69" t="s">
-        <v>2422</v>
+        <v>2397</v>
       </c>
       <c r="O69" t="s">
-        <v>2361</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2801</v>
+      </c>
+      <c r="P69" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>698</v>
       </c>
@@ -14067,13 +14325,16 @@
         <v>701</v>
       </c>
       <c r="N70" t="s">
-        <v>2423</v>
+        <v>2398</v>
       </c>
       <c r="O70" t="s">
-        <v>2362</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2802</v>
+      </c>
+      <c r="P70" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>705</v>
       </c>
@@ -14114,13 +14375,16 @@
         <v>708</v>
       </c>
       <c r="N71" t="s">
-        <v>2424</v>
+        <v>2399</v>
       </c>
       <c r="O71" t="s">
-        <v>2363</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+        <v>2803</v>
+      </c>
+      <c r="P71" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>712</v>
       </c>
@@ -14161,10 +14425,13 @@
         <v>715</v>
       </c>
       <c r="N72" t="s">
-        <v>2425</v>
+        <v>2400</v>
       </c>
       <c r="O72" t="s">
-        <v>2364</v>
+        <v>2804</v>
+      </c>
+      <c r="P72" t="s">
+        <v>713</v>
       </c>
     </row>
   </sheetData>
@@ -14302,13 +14569,13 @@
         <v>727</v>
       </c>
       <c r="N3" t="s">
-        <v>2426</v>
+        <v>2401</v>
       </c>
       <c r="O3" t="s">
-        <v>2429</v>
+        <v>2404</v>
       </c>
       <c r="P3" t="s">
-        <v>2433</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -14374,13 +14641,13 @@
         <v>744</v>
       </c>
       <c r="N6" t="s">
-        <v>2427</v>
+        <v>2402</v>
       </c>
       <c r="O6" t="s">
-        <v>2430</v>
+        <v>2405</v>
       </c>
       <c r="P6" t="s">
-        <v>2434</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -14424,13 +14691,13 @@
         <v>757</v>
       </c>
       <c r="N7" t="s">
-        <v>2428</v>
+        <v>2403</v>
       </c>
       <c r="O7" t="s">
-        <v>2431</v>
+        <v>2406</v>
       </c>
       <c r="P7" t="s">
-        <v>2435</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -14459,7 +14726,7 @@
         <v>763</v>
       </c>
       <c r="O8" t="s">
-        <v>2432</v>
+        <v>2407</v>
       </c>
     </row>
   </sheetData>
@@ -14605,13 +14872,13 @@
         <v>771</v>
       </c>
       <c r="N3" t="s">
-        <v>2436</v>
+        <v>2411</v>
       </c>
       <c r="O3" t="s">
-        <v>2444</v>
+        <v>2419</v>
       </c>
       <c r="P3" t="s">
-        <v>2452</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -14655,13 +14922,13 @@
         <v>784</v>
       </c>
       <c r="N4" t="s">
-        <v>2437</v>
+        <v>2412</v>
       </c>
       <c r="O4" t="s">
-        <v>2445</v>
+        <v>2420</v>
       </c>
       <c r="P4" t="s">
-        <v>2453</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -14705,13 +14972,13 @@
         <v>2213</v>
       </c>
       <c r="N5" t="s">
-        <v>2438</v>
+        <v>2413</v>
       </c>
       <c r="O5" t="s">
-        <v>2446</v>
+        <v>2421</v>
       </c>
       <c r="P5" t="s">
-        <v>2454</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -14755,13 +15022,13 @@
         <v>803</v>
       </c>
       <c r="N6" t="s">
-        <v>2439</v>
+        <v>2414</v>
       </c>
       <c r="O6" t="s">
-        <v>2447</v>
+        <v>2422</v>
       </c>
       <c r="P6" t="s">
-        <v>2455</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -14805,13 +15072,13 @@
         <v>815</v>
       </c>
       <c r="N7" t="s">
-        <v>2440</v>
+        <v>2415</v>
       </c>
       <c r="O7" t="s">
-        <v>2448</v>
+        <v>2423</v>
       </c>
       <c r="P7" t="s">
-        <v>2456</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -14855,13 +15122,13 @@
         <v>827</v>
       </c>
       <c r="N8" t="s">
-        <v>2441</v>
+        <v>2416</v>
       </c>
       <c r="O8" t="s">
-        <v>2449</v>
+        <v>2424</v>
       </c>
       <c r="P8" t="s">
-        <v>2457</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -14905,13 +15172,13 @@
         <v>840</v>
       </c>
       <c r="N9" t="s">
-        <v>2442</v>
+        <v>2417</v>
       </c>
       <c r="O9" t="s">
-        <v>2450</v>
+        <v>2425</v>
       </c>
       <c r="P9" t="s">
-        <v>2458</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -14955,10 +15222,10 @@
         <v>850</v>
       </c>
       <c r="N10" t="s">
-        <v>2443</v>
+        <v>2418</v>
       </c>
       <c r="O10" t="s">
-        <v>2451</v>
+        <v>2426</v>
       </c>
       <c r="P10" t="s">
         <v>846</v>
@@ -15105,13 +15372,13 @@
         <v>862</v>
       </c>
       <c r="N3" t="s">
-        <v>2459</v>
+        <v>2434</v>
       </c>
       <c r="O3" t="s">
-        <v>2463</v>
+        <v>2438</v>
       </c>
       <c r="P3" t="s">
-        <v>2467</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -15155,13 +15422,13 @@
         <v>872</v>
       </c>
       <c r="N4" t="s">
-        <v>2460</v>
+        <v>2435</v>
       </c>
       <c r="O4" t="s">
-        <v>2464</v>
+        <v>2439</v>
       </c>
       <c r="P4" t="s">
-        <v>2468</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -15205,13 +15472,13 @@
         <v>879</v>
       </c>
       <c r="N5" t="s">
-        <v>2461</v>
+        <v>2436</v>
       </c>
       <c r="O5" t="s">
-        <v>2465</v>
+        <v>2440</v>
       </c>
       <c r="P5" t="s">
-        <v>2469</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -15255,13 +15522,13 @@
         <v>887</v>
       </c>
       <c r="N6" t="s">
-        <v>2462</v>
+        <v>2437</v>
       </c>
       <c r="O6" t="s">
-        <v>2466</v>
+        <v>2441</v>
       </c>
       <c r="P6" t="s">
-        <v>2470</v>
+        <v>2445</v>
       </c>
     </row>
   </sheetData>
@@ -15413,13 +15680,13 @@
         <v>899</v>
       </c>
       <c r="O3" t="s">
-        <v>2471</v>
+        <v>2446</v>
       </c>
       <c r="P3" t="s">
-        <v>2473</v>
+        <v>2448</v>
       </c>
       <c r="Q3" t="s">
-        <v>2475</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -15463,13 +15730,13 @@
         <v>909</v>
       </c>
       <c r="O4" t="s">
-        <v>2472</v>
+        <v>2447</v>
       </c>
       <c r="P4" t="s">
-        <v>2474</v>
+        <v>2449</v>
       </c>
       <c r="Q4" t="s">
-        <v>2476</v>
+        <v>2451</v>
       </c>
     </row>
   </sheetData>
@@ -15617,10 +15884,10 @@
         <v>918</v>
       </c>
       <c r="N3" t="s">
-        <v>2477</v>
+        <v>2452</v>
       </c>
       <c r="O3" t="s">
-        <v>2566</v>
+        <v>2541</v>
       </c>
       <c r="P3" t="s">
         <v>914</v>
@@ -15667,10 +15934,10 @@
         <v>928</v>
       </c>
       <c r="N4" t="s">
-        <v>2478</v>
+        <v>2453</v>
       </c>
       <c r="O4" t="s">
-        <v>2567</v>
+        <v>2542</v>
       </c>
       <c r="P4" t="s">
         <v>924</v>
@@ -15717,10 +15984,10 @@
         <v>938</v>
       </c>
       <c r="N5" t="s">
-        <v>2479</v>
+        <v>2454</v>
       </c>
       <c r="O5" t="s">
-        <v>2657</v>
+        <v>2632</v>
       </c>
       <c r="P5" t="s">
         <v>934</v>
@@ -15767,10 +16034,10 @@
         <v>948</v>
       </c>
       <c r="N6" t="s">
-        <v>2480</v>
+        <v>2455</v>
       </c>
       <c r="O6" t="s">
-        <v>2568</v>
+        <v>2543</v>
       </c>
       <c r="P6" t="s">
         <v>944</v>
@@ -15817,10 +16084,10 @@
         <v>958</v>
       </c>
       <c r="N7" t="s">
-        <v>2481</v>
+        <v>2456</v>
       </c>
       <c r="O7" t="s">
-        <v>2569</v>
+        <v>2544</v>
       </c>
       <c r="P7" t="s">
         <v>954</v>
@@ -15867,10 +16134,10 @@
         <v>968</v>
       </c>
       <c r="N8" t="s">
-        <v>2482</v>
+        <v>2457</v>
       </c>
       <c r="O8" t="s">
-        <v>2570</v>
+        <v>2545</v>
       </c>
       <c r="P8" t="s">
         <v>964</v>
@@ -15917,10 +16184,10 @@
         <v>978</v>
       </c>
       <c r="N9" t="s">
-        <v>2483</v>
+        <v>2458</v>
       </c>
       <c r="O9" t="s">
-        <v>2571</v>
+        <v>2546</v>
       </c>
       <c r="P9" t="s">
         <v>974</v>
@@ -15967,10 +16234,10 @@
         <v>988</v>
       </c>
       <c r="N10" t="s">
-        <v>2484</v>
+        <v>2459</v>
       </c>
       <c r="O10" t="s">
-        <v>2572</v>
+        <v>2547</v>
       </c>
       <c r="P10" t="s">
         <v>984</v>
@@ -16017,13 +16284,13 @@
         <v>999</v>
       </c>
       <c r="N11" t="s">
-        <v>2485</v>
+        <v>2460</v>
       </c>
       <c r="O11" t="s">
-        <v>2573</v>
+        <v>2548</v>
       </c>
       <c r="P11" t="s">
-        <v>2658</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -16067,13 +16334,13 @@
         <v>1011</v>
       </c>
       <c r="N12" t="s">
-        <v>2486</v>
+        <v>2461</v>
       </c>
       <c r="O12" t="s">
-        <v>2574</v>
+        <v>2549</v>
       </c>
       <c r="P12" t="s">
-        <v>2659</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -16117,13 +16384,13 @@
         <v>1022</v>
       </c>
       <c r="N13" t="s">
-        <v>2487</v>
+        <v>2462</v>
       </c>
       <c r="O13" t="s">
-        <v>2575</v>
+        <v>2550</v>
       </c>
       <c r="P13" t="s">
-        <v>2660</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -16167,13 +16434,13 @@
         <v>1031</v>
       </c>
       <c r="N14" t="s">
-        <v>2488</v>
+        <v>2463</v>
       </c>
       <c r="O14" t="s">
-        <v>2576</v>
+        <v>2551</v>
       </c>
       <c r="P14" t="s">
-        <v>2661</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -16217,13 +16484,13 @@
         <v>1041</v>
       </c>
       <c r="N15" t="s">
-        <v>2489</v>
+        <v>2464</v>
       </c>
       <c r="O15" t="s">
-        <v>2577</v>
+        <v>2552</v>
       </c>
       <c r="P15" t="s">
-        <v>2662</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -16267,13 +16534,13 @@
         <v>1052</v>
       </c>
       <c r="N16" t="s">
-        <v>2490</v>
+        <v>2465</v>
       </c>
       <c r="O16" t="s">
-        <v>2578</v>
+        <v>2553</v>
       </c>
       <c r="P16" t="s">
-        <v>2663</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -16317,13 +16584,13 @@
         <v>1065</v>
       </c>
       <c r="N17" t="s">
-        <v>2491</v>
+        <v>2466</v>
       </c>
       <c r="O17" t="s">
-        <v>2579</v>
+        <v>2554</v>
       </c>
       <c r="P17" t="s">
-        <v>2664</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -16367,13 +16634,13 @@
         <v>1075</v>
       </c>
       <c r="N18" t="s">
-        <v>2492</v>
+        <v>2467</v>
       </c>
       <c r="O18" t="s">
-        <v>2580</v>
+        <v>2555</v>
       </c>
       <c r="P18" t="s">
-        <v>2665</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -16417,13 +16684,13 @@
         <v>1086</v>
       </c>
       <c r="N19" t="s">
-        <v>2493</v>
+        <v>2468</v>
       </c>
       <c r="O19" t="s">
-        <v>2581</v>
+        <v>2556</v>
       </c>
       <c r="P19" t="s">
-        <v>2666</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -16467,10 +16734,10 @@
         <v>1093</v>
       </c>
       <c r="N20" t="s">
-        <v>2494</v>
+        <v>2469</v>
       </c>
       <c r="O20" t="s">
-        <v>2582</v>
+        <v>2557</v>
       </c>
       <c r="P20" t="s">
         <v>1091</v>
@@ -16517,10 +16784,10 @@
         <v>1105</v>
       </c>
       <c r="N21" t="s">
-        <v>2495</v>
+        <v>2470</v>
       </c>
       <c r="O21" t="s">
-        <v>2583</v>
+        <v>2558</v>
       </c>
       <c r="P21" t="s">
         <v>1098</v>
@@ -16567,13 +16834,13 @@
         <v>1116</v>
       </c>
       <c r="N22" t="s">
-        <v>2496</v>
+        <v>2471</v>
       </c>
       <c r="O22" t="s">
-        <v>2584</v>
+        <v>2559</v>
       </c>
       <c r="P22" t="s">
-        <v>2667</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
@@ -16667,13 +16934,13 @@
         <v>1128</v>
       </c>
       <c r="N24" t="s">
-        <v>2497</v>
+        <v>2472</v>
       </c>
       <c r="O24" t="s">
-        <v>2585</v>
+        <v>2560</v>
       </c>
       <c r="P24" t="s">
-        <v>2668</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
@@ -16717,10 +16984,10 @@
         <v>1138</v>
       </c>
       <c r="N25" t="s">
-        <v>2498</v>
+        <v>2473</v>
       </c>
       <c r="O25" t="s">
-        <v>2586</v>
+        <v>2561</v>
       </c>
       <c r="P25" t="s">
         <v>1136</v>
@@ -16767,13 +17034,13 @@
         <v>1146</v>
       </c>
       <c r="N26" t="s">
-        <v>2499</v>
+        <v>2474</v>
       </c>
       <c r="O26" t="s">
-        <v>2587</v>
+        <v>2562</v>
       </c>
       <c r="P26" t="s">
-        <v>2669</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
@@ -16817,13 +17084,13 @@
         <v>1153</v>
       </c>
       <c r="N27" t="s">
-        <v>2500</v>
+        <v>2475</v>
       </c>
       <c r="O27" t="s">
-        <v>2588</v>
+        <v>2563</v>
       </c>
       <c r="P27" t="s">
-        <v>2670</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
@@ -16867,13 +17134,13 @@
         <v>1161</v>
       </c>
       <c r="N28" t="s">
-        <v>2501</v>
+        <v>2476</v>
       </c>
       <c r="O28" t="s">
-        <v>2589</v>
+        <v>2564</v>
       </c>
       <c r="P28" t="s">
-        <v>2671</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
@@ -16917,10 +17184,10 @@
         <v>1174</v>
       </c>
       <c r="N29" t="s">
-        <v>2502</v>
+        <v>2477</v>
       </c>
       <c r="O29" t="s">
-        <v>2590</v>
+        <v>2565</v>
       </c>
       <c r="P29" t="s">
         <v>1171</v>
@@ -16967,13 +17234,13 @@
         <v>1184</v>
       </c>
       <c r="N30" t="s">
-        <v>2503</v>
+        <v>2478</v>
       </c>
       <c r="O30" t="s">
-        <v>2591</v>
+        <v>2566</v>
       </c>
       <c r="P30" t="s">
-        <v>2672</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.2">
@@ -17017,13 +17284,13 @@
         <v>1194</v>
       </c>
       <c r="N31" t="s">
-        <v>2504</v>
+        <v>2479</v>
       </c>
       <c r="O31" t="s">
-        <v>2592</v>
+        <v>2567</v>
       </c>
       <c r="P31" t="s">
-        <v>2721</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
@@ -17067,10 +17334,10 @@
         <v>1203</v>
       </c>
       <c r="N32" t="s">
-        <v>2505</v>
+        <v>2480</v>
       </c>
       <c r="O32" t="s">
-        <v>2593</v>
+        <v>2568</v>
       </c>
       <c r="P32" t="s">
         <v>1201</v>
@@ -17117,13 +17384,13 @@
         <v>1214</v>
       </c>
       <c r="N33" t="s">
-        <v>2506</v>
+        <v>2481</v>
       </c>
       <c r="O33" t="s">
-        <v>2594</v>
+        <v>2569</v>
       </c>
       <c r="P33" t="s">
-        <v>2673</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.2">
@@ -17167,13 +17434,13 @@
         <v>1221</v>
       </c>
       <c r="N34" t="s">
-        <v>2507</v>
+        <v>2482</v>
       </c>
       <c r="O34" t="s">
-        <v>2595</v>
+        <v>2570</v>
       </c>
       <c r="P34" t="s">
-        <v>2674</v>
+        <v>2649</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.2">
@@ -17217,13 +17484,13 @@
         <v>1233</v>
       </c>
       <c r="N35" t="s">
-        <v>2508</v>
+        <v>2483</v>
       </c>
       <c r="O35" t="s">
-        <v>2596</v>
+        <v>2571</v>
       </c>
       <c r="P35" t="s">
-        <v>2675</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
@@ -17267,10 +17534,10 @@
         <v>1243</v>
       </c>
       <c r="N36" t="s">
-        <v>2509</v>
+        <v>2484</v>
       </c>
       <c r="O36" t="s">
-        <v>2597</v>
+        <v>2572</v>
       </c>
       <c r="P36" t="s">
         <v>1239</v>
@@ -17317,13 +17584,13 @@
         <v>1255</v>
       </c>
       <c r="N37" t="s">
-        <v>2510</v>
+        <v>2485</v>
       </c>
       <c r="O37" t="s">
-        <v>2598</v>
+        <v>2573</v>
       </c>
       <c r="P37" t="s">
-        <v>2676</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
@@ -17367,13 +17634,13 @@
         <v>1267</v>
       </c>
       <c r="N38" t="s">
-        <v>2511</v>
+        <v>2486</v>
       </c>
       <c r="O38" t="s">
-        <v>2599</v>
+        <v>2574</v>
       </c>
       <c r="P38" t="s">
-        <v>2677</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
@@ -17417,13 +17684,13 @@
         <v>1275</v>
       </c>
       <c r="N39" t="s">
-        <v>2512</v>
+        <v>2487</v>
       </c>
       <c r="O39" t="s">
-        <v>2600</v>
+        <v>2575</v>
       </c>
       <c r="P39" t="s">
-        <v>2678</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.2">
@@ -17470,10 +17737,10 @@
         <v>1287</v>
       </c>
       <c r="O40" t="s">
-        <v>2601</v>
+        <v>2576</v>
       </c>
       <c r="P40" t="s">
-        <v>2679</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.2">
@@ -17517,13 +17784,13 @@
         <v>1298</v>
       </c>
       <c r="N41" t="s">
-        <v>2513</v>
+        <v>2488</v>
       </c>
       <c r="O41" t="s">
-        <v>2602</v>
+        <v>2577</v>
       </c>
       <c r="P41" t="s">
-        <v>2680</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.2">
@@ -17567,13 +17834,13 @@
         <v>1310</v>
       </c>
       <c r="N42" t="s">
-        <v>2514</v>
+        <v>2489</v>
       </c>
       <c r="O42" t="s">
-        <v>2603</v>
+        <v>2578</v>
       </c>
       <c r="P42" t="s">
-        <v>2681</v>
+        <v>2656</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.2">
@@ -17617,13 +17884,13 @@
         <v>1320</v>
       </c>
       <c r="N43" t="s">
-        <v>2515</v>
+        <v>2490</v>
       </c>
       <c r="O43" t="s">
-        <v>2604</v>
+        <v>2579</v>
       </c>
       <c r="P43" t="s">
-        <v>2682</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.2">
@@ -17667,13 +17934,13 @@
         <v>1331</v>
       </c>
       <c r="N44" t="s">
-        <v>2516</v>
+        <v>2491</v>
       </c>
       <c r="O44" t="s">
-        <v>2605</v>
+        <v>2580</v>
       </c>
       <c r="P44" t="s">
-        <v>2683</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.2">
@@ -17717,13 +17984,13 @@
         <v>1341</v>
       </c>
       <c r="N45" t="s">
-        <v>2517</v>
+        <v>2492</v>
       </c>
       <c r="O45" t="s">
-        <v>2606</v>
+        <v>2581</v>
       </c>
       <c r="P45" t="s">
-        <v>2684</v>
+        <v>2659</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.2">
@@ -17817,10 +18084,10 @@
         <v>1350</v>
       </c>
       <c r="N47" t="s">
-        <v>2518</v>
+        <v>2493</v>
       </c>
       <c r="O47" t="s">
-        <v>2607</v>
+        <v>2582</v>
       </c>
       <c r="P47" t="s">
         <v>1351</v>
@@ -17867,13 +18134,13 @@
         <v>1362</v>
       </c>
       <c r="N48" t="s">
-        <v>2519</v>
+        <v>2494</v>
       </c>
       <c r="O48" t="s">
-        <v>2608</v>
+        <v>2583</v>
       </c>
       <c r="P48" t="s">
-        <v>2685</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
@@ -17917,10 +18184,10 @@
         <v>1372</v>
       </c>
       <c r="N49" t="s">
-        <v>2520</v>
+        <v>2495</v>
       </c>
       <c r="O49" t="s">
-        <v>2609</v>
+        <v>2584</v>
       </c>
       <c r="P49" t="s">
         <v>1368</v>
@@ -17970,7 +18237,7 @@
         <v>1378</v>
       </c>
       <c r="O50" t="s">
-        <v>2610</v>
+        <v>2585</v>
       </c>
       <c r="P50" t="s">
         <v>1376</v>
@@ -18017,13 +18284,13 @@
         <v>1390</v>
       </c>
       <c r="N51" t="s">
-        <v>2521</v>
+        <v>2496</v>
       </c>
       <c r="O51" t="s">
-        <v>2611</v>
+        <v>2586</v>
       </c>
       <c r="P51" t="s">
-        <v>2686</v>
+        <v>2661</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.2">
@@ -18067,13 +18334,13 @@
         <v>1401</v>
       </c>
       <c r="N52" t="s">
-        <v>2522</v>
+        <v>2497</v>
       </c>
       <c r="O52" t="s">
-        <v>2612</v>
+        <v>2587</v>
       </c>
       <c r="P52" t="s">
-        <v>2687</v>
+        <v>2662</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.2">
@@ -18117,13 +18384,13 @@
         <v>1409</v>
       </c>
       <c r="N53" t="s">
-        <v>2523</v>
+        <v>2498</v>
       </c>
       <c r="O53" t="s">
-        <v>2613</v>
+        <v>2588</v>
       </c>
       <c r="P53" t="s">
-        <v>2688</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.2">
@@ -18167,10 +18434,10 @@
         <v>1417</v>
       </c>
       <c r="N54" t="s">
-        <v>2524</v>
+        <v>2499</v>
       </c>
       <c r="O54" t="s">
-        <v>2614</v>
+        <v>2589</v>
       </c>
       <c r="P54" t="s">
         <v>1415</v>
@@ -18217,13 +18484,13 @@
         <v>1429</v>
       </c>
       <c r="N55" t="s">
-        <v>2525</v>
+        <v>2500</v>
       </c>
       <c r="O55" t="s">
-        <v>2615</v>
+        <v>2590</v>
       </c>
       <c r="P55" t="s">
-        <v>2689</v>
+        <v>2664</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.2">
@@ -18267,13 +18534,13 @@
         <v>1439</v>
       </c>
       <c r="N56" t="s">
-        <v>2526</v>
+        <v>2501</v>
       </c>
       <c r="O56" t="s">
-        <v>2616</v>
+        <v>2591</v>
       </c>
       <c r="P56" t="s">
-        <v>2690</v>
+        <v>2665</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.2">
@@ -18317,13 +18584,13 @@
         <v>1449</v>
       </c>
       <c r="N57" t="s">
-        <v>2527</v>
+        <v>2502</v>
       </c>
       <c r="O57" t="s">
-        <v>2617</v>
+        <v>2592</v>
       </c>
       <c r="P57" t="s">
-        <v>2691</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.2">
@@ -18367,13 +18634,13 @@
         <v>1161</v>
       </c>
       <c r="N58" t="s">
-        <v>2501</v>
+        <v>2476</v>
       </c>
       <c r="O58" t="s">
-        <v>2589</v>
+        <v>2564</v>
       </c>
       <c r="P58" t="s">
-        <v>2671</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.2">
@@ -18417,10 +18684,10 @@
         <v>1462</v>
       </c>
       <c r="N59" t="s">
-        <v>2528</v>
+        <v>2503</v>
       </c>
       <c r="O59" t="s">
-        <v>2618</v>
+        <v>2593</v>
       </c>
       <c r="P59" t="s">
         <v>1460</v>
@@ -18467,13 +18734,13 @@
         <v>1473</v>
       </c>
       <c r="N60" t="s">
-        <v>2529</v>
+        <v>2504</v>
       </c>
       <c r="O60" t="s">
-        <v>2619</v>
+        <v>2594</v>
       </c>
       <c r="P60" t="s">
-        <v>2692</v>
+        <v>2667</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.2">
@@ -18517,13 +18784,13 @@
         <v>1484</v>
       </c>
       <c r="N61" t="s">
-        <v>2530</v>
+        <v>2505</v>
       </c>
       <c r="O61" t="s">
-        <v>2620</v>
+        <v>2595</v>
       </c>
       <c r="P61" t="s">
-        <v>2693</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.2">
@@ -18567,13 +18834,13 @@
         <v>1495</v>
       </c>
       <c r="N62" t="s">
-        <v>2531</v>
+        <v>2506</v>
       </c>
       <c r="O62" t="s">
-        <v>2621</v>
+        <v>2596</v>
       </c>
       <c r="P62" t="s">
-        <v>2694</v>
+        <v>2669</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.2">
@@ -18667,10 +18934,10 @@
         <v>1504</v>
       </c>
       <c r="N64" t="s">
-        <v>2532</v>
+        <v>2507</v>
       </c>
       <c r="O64" t="s">
-        <v>2622</v>
+        <v>2597</v>
       </c>
       <c r="P64" t="s">
         <v>1502</v>
@@ -18717,13 +18984,13 @@
         <v>1515</v>
       </c>
       <c r="N65" t="s">
-        <v>2533</v>
+        <v>2508</v>
       </c>
       <c r="O65" t="s">
-        <v>2623</v>
+        <v>2598</v>
       </c>
       <c r="P65" t="s">
-        <v>2695</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.2">
@@ -18767,13 +19034,13 @@
         <v>1525</v>
       </c>
       <c r="N66" t="s">
-        <v>2534</v>
+        <v>2509</v>
       </c>
       <c r="O66" t="s">
-        <v>2624</v>
+        <v>2599</v>
       </c>
       <c r="P66" t="s">
-        <v>2696</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.2">
@@ -18817,13 +19084,13 @@
         <v>1532</v>
       </c>
       <c r="N67" t="s">
-        <v>2535</v>
+        <v>2510</v>
       </c>
       <c r="O67" t="s">
-        <v>2625</v>
+        <v>2600</v>
       </c>
       <c r="P67" t="s">
-        <v>2697</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.2">
@@ -18867,13 +19134,13 @@
         <v>1544</v>
       </c>
       <c r="N68" t="s">
-        <v>2536</v>
+        <v>2511</v>
       </c>
       <c r="O68" t="s">
-        <v>2626</v>
+        <v>2601</v>
       </c>
       <c r="P68" t="s">
-        <v>2698</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.2">
@@ -18917,13 +19184,13 @@
         <v>1552</v>
       </c>
       <c r="N69" t="s">
-        <v>2537</v>
+        <v>2512</v>
       </c>
       <c r="O69" t="s">
-        <v>2627</v>
+        <v>2602</v>
       </c>
       <c r="P69" t="s">
-        <v>2699</v>
+        <v>2674</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.2">
@@ -18967,13 +19234,13 @@
         <v>1565</v>
       </c>
       <c r="N70" t="s">
-        <v>2538</v>
+        <v>2513</v>
       </c>
       <c r="O70" t="s">
-        <v>2628</v>
+        <v>2603</v>
       </c>
       <c r="P70" t="s">
-        <v>2700</v>
+        <v>2675</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.2">
@@ -19017,13 +19284,13 @@
         <v>1578</v>
       </c>
       <c r="N71" t="s">
-        <v>2539</v>
+        <v>2514</v>
       </c>
       <c r="O71" t="s">
-        <v>2629</v>
+        <v>2604</v>
       </c>
       <c r="P71" t="s">
-        <v>2701</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.2">
@@ -19067,13 +19334,13 @@
         <v>1591</v>
       </c>
       <c r="N72" t="s">
-        <v>2540</v>
+        <v>2515</v>
       </c>
       <c r="O72" t="s">
-        <v>2630</v>
+        <v>2605</v>
       </c>
       <c r="P72" t="s">
-        <v>2702</v>
+        <v>2677</v>
       </c>
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.2">
@@ -19117,13 +19384,13 @@
         <v>1602</v>
       </c>
       <c r="N73" t="s">
-        <v>2541</v>
+        <v>2516</v>
       </c>
       <c r="O73" t="s">
-        <v>2631</v>
+        <v>2606</v>
       </c>
       <c r="P73" t="s">
-        <v>2703</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.2">
@@ -19167,10 +19434,10 @@
         <v>1611</v>
       </c>
       <c r="N74" t="s">
-        <v>2542</v>
+        <v>2517</v>
       </c>
       <c r="O74" t="s">
-        <v>2632</v>
+        <v>2607</v>
       </c>
       <c r="P74" t="s">
         <v>1608</v>
@@ -19217,10 +19484,10 @@
         <v>1618</v>
       </c>
       <c r="N75" t="s">
-        <v>2543</v>
+        <v>2518</v>
       </c>
       <c r="O75" t="s">
-        <v>2633</v>
+        <v>2608</v>
       </c>
       <c r="P75" t="s">
         <v>1616</v>
@@ -19267,10 +19534,10 @@
         <v>1628</v>
       </c>
       <c r="N76" t="s">
-        <v>2544</v>
+        <v>2519</v>
       </c>
       <c r="O76" t="s">
-        <v>2634</v>
+        <v>2609</v>
       </c>
       <c r="P76" t="s">
         <v>1623</v>
@@ -19317,13 +19584,13 @@
         <v>1639</v>
       </c>
       <c r="N77" t="s">
-        <v>2545</v>
+        <v>2520</v>
       </c>
       <c r="O77" t="s">
-        <v>2635</v>
+        <v>2610</v>
       </c>
       <c r="P77" t="s">
-        <v>2704</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.2">
@@ -19367,13 +19634,13 @@
         <v>1649</v>
       </c>
       <c r="N78" t="s">
-        <v>2546</v>
+        <v>2521</v>
       </c>
       <c r="O78" t="s">
-        <v>2636</v>
+        <v>2611</v>
       </c>
       <c r="P78" t="s">
-        <v>2705</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.2">
@@ -19417,13 +19684,13 @@
         <v>1658</v>
       </c>
       <c r="N79" t="s">
-        <v>2547</v>
+        <v>2522</v>
       </c>
       <c r="O79" t="s">
-        <v>2637</v>
+        <v>2612</v>
       </c>
       <c r="P79" t="s">
-        <v>2706</v>
+        <v>2681</v>
       </c>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.2">
@@ -19517,13 +19784,13 @@
         <v>1669</v>
       </c>
       <c r="N81" t="s">
-        <v>2548</v>
+        <v>2523</v>
       </c>
       <c r="O81" t="s">
-        <v>2638</v>
+        <v>2613</v>
       </c>
       <c r="P81" t="s">
-        <v>2707</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.2">
@@ -19617,13 +19884,13 @@
         <v>1683</v>
       </c>
       <c r="N83" t="s">
-        <v>2549</v>
+        <v>2524</v>
       </c>
       <c r="O83" t="s">
-        <v>2639</v>
+        <v>2614</v>
       </c>
       <c r="P83" t="s">
-        <v>2708</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.2">
@@ -19667,13 +19934,13 @@
         <v>1695</v>
       </c>
       <c r="N84" t="s">
-        <v>2550</v>
+        <v>2525</v>
       </c>
       <c r="O84" t="s">
-        <v>2640</v>
+        <v>2615</v>
       </c>
       <c r="P84" t="s">
-        <v>2709</v>
+        <v>2684</v>
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.2">
@@ -19717,10 +19984,10 @@
         <v>1704</v>
       </c>
       <c r="N85" t="s">
-        <v>2551</v>
+        <v>2526</v>
       </c>
       <c r="O85" t="s">
-        <v>2641</v>
+        <v>2616</v>
       </c>
       <c r="P85" t="s">
         <v>1701</v>
@@ -19767,13 +20034,13 @@
         <v>1714</v>
       </c>
       <c r="N86" t="s">
-        <v>2552</v>
+        <v>2527</v>
       </c>
       <c r="O86" t="s">
-        <v>2642</v>
+        <v>2617</v>
       </c>
       <c r="P86" t="s">
-        <v>2710</v>
+        <v>2685</v>
       </c>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.2">
@@ -19817,13 +20084,13 @@
         <v>1727</v>
       </c>
       <c r="N87" t="s">
-        <v>2553</v>
+        <v>2528</v>
       </c>
       <c r="O87" t="s">
-        <v>2643</v>
+        <v>2618</v>
       </c>
       <c r="P87" t="s">
-        <v>2711</v>
+        <v>2686</v>
       </c>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.2">
@@ -19867,13 +20134,13 @@
         <v>1739</v>
       </c>
       <c r="N88" t="s">
-        <v>2554</v>
+        <v>2529</v>
       </c>
       <c r="O88" t="s">
-        <v>2644</v>
+        <v>2619</v>
       </c>
       <c r="P88" t="s">
-        <v>2712</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.2">
@@ -19917,13 +20184,13 @@
         <v>1750</v>
       </c>
       <c r="N89" t="s">
-        <v>2555</v>
+        <v>2530</v>
       </c>
       <c r="O89" t="s">
-        <v>2645</v>
+        <v>2620</v>
       </c>
       <c r="P89" t="s">
-        <v>2713</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.2">
@@ -19967,13 +20234,13 @@
         <v>1763</v>
       </c>
       <c r="N90" t="s">
-        <v>2556</v>
+        <v>2531</v>
       </c>
       <c r="O90" t="s">
-        <v>2646</v>
+        <v>2621</v>
       </c>
       <c r="P90" t="s">
-        <v>2714</v>
+        <v>2689</v>
       </c>
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.2">
@@ -20020,10 +20287,10 @@
         <v>1774</v>
       </c>
       <c r="O91" t="s">
-        <v>2647</v>
+        <v>2622</v>
       </c>
       <c r="P91" t="s">
-        <v>2715</v>
+        <v>2690</v>
       </c>
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.2">
@@ -20067,10 +20334,10 @@
         <v>1787</v>
       </c>
       <c r="N92" t="s">
-        <v>2557</v>
+        <v>2532</v>
       </c>
       <c r="O92" t="s">
-        <v>2648</v>
+        <v>2623</v>
       </c>
       <c r="P92" t="s">
         <v>1780</v>
@@ -20117,13 +20384,13 @@
         <v>1799</v>
       </c>
       <c r="N93" t="s">
-        <v>2558</v>
+        <v>2533</v>
       </c>
       <c r="O93" t="s">
-        <v>2649</v>
+        <v>2624</v>
       </c>
       <c r="P93" t="s">
-        <v>2716</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="94" spans="1:16" x14ac:dyDescent="0.2">
@@ -20167,13 +20434,13 @@
         <v>1810</v>
       </c>
       <c r="N94" t="s">
-        <v>2559</v>
+        <v>2534</v>
       </c>
       <c r="O94" t="s">
-        <v>2650</v>
+        <v>2625</v>
       </c>
       <c r="P94" t="s">
-        <v>2717</v>
+        <v>2692</v>
       </c>
     </row>
     <row r="95" spans="1:16" x14ac:dyDescent="0.2">
@@ -20217,10 +20484,10 @@
         <v>1818</v>
       </c>
       <c r="N95" t="s">
-        <v>2560</v>
+        <v>2535</v>
       </c>
       <c r="O95" t="s">
-        <v>2651</v>
+        <v>2626</v>
       </c>
       <c r="P95" t="s">
         <v>1816</v>
@@ -20317,13 +20584,13 @@
         <v>1833</v>
       </c>
       <c r="N97" t="s">
-        <v>2561</v>
+        <v>2536</v>
       </c>
       <c r="O97" t="s">
-        <v>2652</v>
+        <v>2627</v>
       </c>
       <c r="P97" t="s">
-        <v>2718</v>
+        <v>2693</v>
       </c>
     </row>
     <row r="98" spans="1:16" x14ac:dyDescent="0.2">
@@ -20367,10 +20634,10 @@
         <v>1841</v>
       </c>
       <c r="N98" t="s">
-        <v>2562</v>
+        <v>2537</v>
       </c>
       <c r="O98" t="s">
-        <v>2653</v>
+        <v>2628</v>
       </c>
       <c r="P98" t="s">
         <v>1839</v>
@@ -20417,10 +20684,10 @@
         <v>1848</v>
       </c>
       <c r="N99" t="s">
-        <v>2563</v>
+        <v>2538</v>
       </c>
       <c r="O99" t="s">
-        <v>2654</v>
+        <v>2629</v>
       </c>
       <c r="P99" t="s">
         <v>1846</v>
@@ -20467,13 +20734,13 @@
         <v>1858</v>
       </c>
       <c r="N100" t="s">
-        <v>2564</v>
+        <v>2539</v>
       </c>
       <c r="O100" t="s">
-        <v>2655</v>
+        <v>2630</v>
       </c>
       <c r="P100" t="s">
-        <v>2719</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="101" spans="1:16" x14ac:dyDescent="0.2">
@@ -20517,13 +20784,13 @@
         <v>1868</v>
       </c>
       <c r="N101" t="s">
-        <v>2565</v>
+        <v>2540</v>
       </c>
       <c r="O101" t="s">
-        <v>2656</v>
+        <v>2631</v>
       </c>
       <c r="P101" t="s">
-        <v>2720</v>
+        <v>2695</v>
       </c>
     </row>
   </sheetData>
@@ -20671,10 +20938,10 @@
         <v>1876</v>
       </c>
       <c r="N3" t="s">
-        <v>2722</v>
+        <v>2697</v>
       </c>
       <c r="O3" t="s">
-        <v>2753</v>
+        <v>2728</v>
       </c>
       <c r="P3" t="s">
         <v>1874</v>
@@ -20721,10 +20988,10 @@
         <v>1883</v>
       </c>
       <c r="N4" t="s">
-        <v>2723</v>
+        <v>2698</v>
       </c>
       <c r="O4" t="s">
-        <v>2754</v>
+        <v>2729</v>
       </c>
       <c r="P4" t="s">
         <v>1880</v>
@@ -20771,13 +21038,13 @@
         <v>1891</v>
       </c>
       <c r="N5" t="s">
-        <v>2724</v>
+        <v>2699</v>
       </c>
       <c r="O5" t="s">
-        <v>2755</v>
+        <v>2730</v>
       </c>
       <c r="P5" t="s">
-        <v>2785</v>
+        <v>2760</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -20821,10 +21088,10 @@
         <v>1898</v>
       </c>
       <c r="N6" t="s">
-        <v>2725</v>
+        <v>2700</v>
       </c>
       <c r="O6" t="s">
-        <v>2756</v>
+        <v>2731</v>
       </c>
       <c r="P6" t="s">
         <v>1895</v>
@@ -20871,10 +21138,10 @@
         <v>1906</v>
       </c>
       <c r="N7" t="s">
-        <v>2726</v>
+        <v>2701</v>
       </c>
       <c r="O7" t="s">
-        <v>2757</v>
+        <v>2732</v>
       </c>
       <c r="P7" t="s">
         <v>1903</v>
@@ -20921,10 +21188,10 @@
         <v>1916</v>
       </c>
       <c r="N8" t="s">
-        <v>2727</v>
+        <v>2702</v>
       </c>
       <c r="O8" t="s">
-        <v>2758</v>
+        <v>2733</v>
       </c>
       <c r="P8" t="s">
         <v>1912</v>
@@ -20971,10 +21238,10 @@
         <v>1923</v>
       </c>
       <c r="N9" t="s">
-        <v>2728</v>
+        <v>2703</v>
       </c>
       <c r="O9" t="s">
-        <v>2759</v>
+        <v>2734</v>
       </c>
       <c r="P9" t="s">
         <v>1921</v>
@@ -21021,10 +21288,10 @@
         <v>1933</v>
       </c>
       <c r="N10" t="s">
-        <v>2729</v>
+        <v>2704</v>
       </c>
       <c r="O10" t="s">
-        <v>2760</v>
+        <v>2735</v>
       </c>
       <c r="P10" t="s">
         <v>1927</v>
@@ -21071,13 +21338,13 @@
         <v>1944</v>
       </c>
       <c r="N11" t="s">
-        <v>2730</v>
+        <v>2705</v>
       </c>
       <c r="O11" t="s">
+        <v>2736</v>
+      </c>
+      <c r="P11" t="s">
         <v>2761</v>
-      </c>
-      <c r="P11" t="s">
-        <v>2786</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -21121,10 +21388,10 @@
         <v>1956</v>
       </c>
       <c r="N12" t="s">
-        <v>2731</v>
+        <v>2706</v>
       </c>
       <c r="O12" t="s">
-        <v>2762</v>
+        <v>2737</v>
       </c>
       <c r="P12" t="s">
         <v>1949</v>
@@ -21171,10 +21438,10 @@
         <v>1964</v>
       </c>
       <c r="N13" t="s">
-        <v>2732</v>
+        <v>2707</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>2763</v>
+        <v>2738</v>
       </c>
       <c r="P13" t="s">
         <v>1961</v>
@@ -21221,10 +21488,10 @@
         <v>1970</v>
       </c>
       <c r="N14" t="s">
-        <v>2733</v>
+        <v>2708</v>
       </c>
       <c r="O14" t="s">
-        <v>2764</v>
+        <v>2739</v>
       </c>
       <c r="P14" t="s">
         <v>1968</v>
@@ -21271,10 +21538,10 @@
         <v>1977</v>
       </c>
       <c r="N15" t="s">
-        <v>2734</v>
+        <v>2709</v>
       </c>
       <c r="O15" t="s">
-        <v>2765</v>
+        <v>2740</v>
       </c>
       <c r="P15" t="s">
         <v>1974</v>
@@ -21321,10 +21588,10 @@
         <v>1986</v>
       </c>
       <c r="N16" t="s">
-        <v>2735</v>
+        <v>2710</v>
       </c>
       <c r="O16" t="s">
-        <v>2766</v>
+        <v>2741</v>
       </c>
       <c r="P16" t="s">
         <v>1982</v>
@@ -21371,10 +21638,10 @@
         <v>1993</v>
       </c>
       <c r="N17" t="s">
-        <v>2736</v>
+        <v>2711</v>
       </c>
       <c r="O17" t="s">
-        <v>2767</v>
+        <v>2742</v>
       </c>
       <c r="P17" t="s">
         <v>1991</v>
@@ -21421,10 +21688,10 @@
         <v>2003</v>
       </c>
       <c r="N18" t="s">
-        <v>2737</v>
+        <v>2712</v>
       </c>
       <c r="O18" t="s">
-        <v>2768</v>
+        <v>2743</v>
       </c>
       <c r="P18" t="s">
         <v>1998</v>
@@ -21471,10 +21738,10 @@
         <v>2013</v>
       </c>
       <c r="N19" t="s">
-        <v>2738</v>
+        <v>2713</v>
       </c>
       <c r="O19" t="s">
-        <v>2769</v>
+        <v>2744</v>
       </c>
       <c r="P19" t="s">
         <v>2008</v>
@@ -21521,10 +21788,10 @@
         <v>2024</v>
       </c>
       <c r="N20" t="s">
-        <v>2739</v>
+        <v>2714</v>
       </c>
       <c r="O20" t="s">
-        <v>2770</v>
+        <v>2745</v>
       </c>
       <c r="P20" t="s">
         <v>2017</v>
@@ -21571,7 +21838,7 @@
         <v>339</v>
       </c>
       <c r="N21" t="s">
-        <v>2383</v>
+        <v>2358</v>
       </c>
       <c r="O21" t="s">
         <v>2316</v>
@@ -21621,10 +21888,10 @@
         <v>2037</v>
       </c>
       <c r="N22" t="s">
-        <v>2740</v>
+        <v>2715</v>
       </c>
       <c r="O22" t="s">
-        <v>2771</v>
+        <v>2746</v>
       </c>
       <c r="P22" t="s">
         <v>2033</v>
@@ -21671,10 +21938,10 @@
         <v>2046</v>
       </c>
       <c r="N23" t="s">
-        <v>2741</v>
+        <v>2716</v>
       </c>
       <c r="O23" t="s">
-        <v>2772</v>
+        <v>2747</v>
       </c>
       <c r="P23" t="s">
         <v>2043</v>
@@ -21721,10 +21988,10 @@
         <v>2053</v>
       </c>
       <c r="N24" t="s">
-        <v>2742</v>
+        <v>2717</v>
       </c>
       <c r="O24" t="s">
-        <v>2773</v>
+        <v>2748</v>
       </c>
       <c r="P24" t="s">
         <v>2051</v>
@@ -21771,10 +22038,10 @@
         <v>2059</v>
       </c>
       <c r="N25" t="s">
-        <v>2743</v>
+        <v>2718</v>
       </c>
       <c r="O25" t="s">
-        <v>2774</v>
+        <v>2749</v>
       </c>
       <c r="P25" t="s">
         <v>2057</v>
@@ -21821,10 +22088,10 @@
         <v>2253</v>
       </c>
       <c r="N26" t="s">
-        <v>2744</v>
+        <v>2719</v>
       </c>
       <c r="O26" t="s">
-        <v>2775</v>
+        <v>2750</v>
       </c>
       <c r="P26" t="s">
         <v>2062</v>
@@ -21871,10 +22138,10 @@
         <v>2078</v>
       </c>
       <c r="N27" t="s">
-        <v>2745</v>
+        <v>2720</v>
       </c>
       <c r="O27" t="s">
-        <v>2776</v>
+        <v>2751</v>
       </c>
       <c r="P27" t="s">
         <v>2074</v>
@@ -21921,13 +22188,13 @@
         <v>2084</v>
       </c>
       <c r="N28" t="s">
-        <v>2746</v>
+        <v>2721</v>
       </c>
       <c r="O28" t="s">
-        <v>2777</v>
+        <v>2752</v>
       </c>
       <c r="P28" t="s">
-        <v>2787</v>
+        <v>2762</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
@@ -21971,13 +22238,13 @@
         <v>2093</v>
       </c>
       <c r="N29" t="s">
-        <v>2747</v>
+        <v>2722</v>
       </c>
       <c r="O29" t="s">
-        <v>2778</v>
+        <v>2753</v>
       </c>
       <c r="P29" t="s">
-        <v>2788</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
@@ -22021,10 +22288,10 @@
         <v>2100</v>
       </c>
       <c r="N30" t="s">
-        <v>2748</v>
+        <v>2723</v>
       </c>
       <c r="O30" t="s">
-        <v>2779</v>
+        <v>2754</v>
       </c>
       <c r="P30" t="s">
         <v>2097</v>
@@ -22071,10 +22338,10 @@
         <v>2110</v>
       </c>
       <c r="N31" t="s">
-        <v>2749</v>
+        <v>2724</v>
       </c>
       <c r="O31" t="s">
-        <v>2780</v>
+        <v>2755</v>
       </c>
       <c r="P31" t="s">
         <v>2105</v>
@@ -22124,10 +22391,10 @@
         <v>2118</v>
       </c>
       <c r="O32" t="s">
-        <v>2781</v>
+        <v>2756</v>
       </c>
       <c r="P32" t="s">
-        <v>2789</v>
+        <v>2764</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.2">
@@ -22171,10 +22438,10 @@
         <v>2126</v>
       </c>
       <c r="N33" t="s">
-        <v>2750</v>
+        <v>2725</v>
       </c>
       <c r="O33" t="s">
-        <v>2782</v>
+        <v>2757</v>
       </c>
       <c r="P33" t="s">
         <v>2123</v>
@@ -22221,10 +22488,10 @@
         <v>2136</v>
       </c>
       <c r="N34" t="s">
-        <v>2751</v>
+        <v>2726</v>
       </c>
       <c r="O34" t="s">
-        <v>2783</v>
+        <v>2758</v>
       </c>
       <c r="P34" t="s">
         <v>2130</v>
@@ -22271,10 +22538,10 @@
         <v>2144</v>
       </c>
       <c r="N35" t="s">
-        <v>2752</v>
+        <v>2727</v>
       </c>
       <c r="O35" t="s">
-        <v>2784</v>
+        <v>2759</v>
       </c>
       <c r="P35" t="s">
         <v>2141</v>
@@ -22321,10 +22588,10 @@
         <v>958</v>
       </c>
       <c r="N36" t="s">
-        <v>2481</v>
+        <v>2456</v>
       </c>
       <c r="O36" t="s">
-        <v>2569</v>
+        <v>2544</v>
       </c>
       <c r="P36" t="s">
         <v>954</v>
@@ -22371,10 +22638,10 @@
         <v>968</v>
       </c>
       <c r="N37" t="s">
-        <v>2482</v>
+        <v>2457</v>
       </c>
       <c r="O37" t="s">
-        <v>2570</v>
+        <v>2545</v>
       </c>
       <c r="P37" t="s">
         <v>964</v>
@@ -22421,10 +22688,10 @@
         <v>978</v>
       </c>
       <c r="N38" t="s">
-        <v>2483</v>
+        <v>2458</v>
       </c>
       <c r="O38" t="s">
-        <v>2571</v>
+        <v>2546</v>
       </c>
       <c r="P38" t="s">
         <v>974</v>
@@ -22471,10 +22738,10 @@
         <v>988</v>
       </c>
       <c r="N39" t="s">
-        <v>2484</v>
+        <v>2459</v>
       </c>
       <c r="O39" t="s">
-        <v>2572</v>
+        <v>2547</v>
       </c>
       <c r="P39" t="s">
         <v>984</v>
@@ -22521,10 +22788,10 @@
         <v>918</v>
       </c>
       <c r="N40" t="s">
-        <v>2477</v>
+        <v>2452</v>
       </c>
       <c r="O40" t="s">
-        <v>2566</v>
+        <v>2541</v>
       </c>
       <c r="P40" t="s">
         <v>914</v>
@@ -22571,10 +22838,10 @@
         <v>928</v>
       </c>
       <c r="N41" t="s">
-        <v>2478</v>
+        <v>2453</v>
       </c>
       <c r="O41" t="s">
-        <v>2567</v>
+        <v>2542</v>
       </c>
       <c r="P41" t="s">
         <v>924</v>
@@ -22621,10 +22888,10 @@
         <v>938</v>
       </c>
       <c r="N42" t="s">
-        <v>2479</v>
+        <v>2454</v>
       </c>
       <c r="O42" t="s">
-        <v>2657</v>
+        <v>2632</v>
       </c>
       <c r="P42" t="s">
         <v>934</v>
@@ -22671,10 +22938,10 @@
         <v>948</v>
       </c>
       <c r="N43" t="s">
-        <v>2480</v>
+        <v>2455</v>
       </c>
       <c r="O43" t="s">
-        <v>2568</v>
+        <v>2543</v>
       </c>
       <c r="P43" t="s">
         <v>944</v>

</xml_diff>

<commit_message>
blank spots for 8 new languages
</commit_message>
<xml_diff>
--- a/src/stp/database/localization.xlsx
+++ b/src/stp/database/localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF29C63-279E-9E46-B3D5-FE0F306AA645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35486CF-AEDC-B046-9067-639E827FE6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Competition" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4256" uniqueCount="2809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4328" uniqueCount="2817">
   <si>
     <t>key</t>
   </si>
@@ -8456,6 +8456,30 @@
   </si>
   <si>
     <t>«Эдьюкейшн сити»</t>
+  </si>
+  <si>
+    <t>el</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>sv</t>
+  </si>
+  <si>
+    <t>cs</t>
+  </si>
+  <si>
+    <t>hr</t>
+  </si>
+  <si>
+    <t>pl</t>
+  </si>
+  <si>
+    <t>sw</t>
+  </si>
+  <si>
+    <t>uz</t>
   </si>
 </sst>
 </file>
@@ -8654,9 +8678,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61B4B980-FFEE-EE4C-9CEC-8AB2B28241C9}" name="Table1" displayName="Table1" ref="A2:P7" totalsRowShown="0">
-  <autoFilter ref="A2:P7" xr:uid="{61B4B980-FFEE-EE4C-9CEC-8AB2B28241C9}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61B4B980-FFEE-EE4C-9CEC-8AB2B28241C9}" name="Table1" displayName="Table1" ref="A2:X7" totalsRowShown="0">
+  <autoFilter ref="A2:X7" xr:uid="{61B4B980-FFEE-EE4C-9CEC-8AB2B28241C9}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{129D1AE6-FFF0-514E-8708-66943724AB60}" name="key"/>
     <tableColumn id="2" xr3:uid="{C21AC7CE-7330-5442-99F9-98294B00509A}" name="en"/>
     <tableColumn id="3" xr3:uid="{4A7EB9F1-733B-3E4F-82FD-0F371C89F290}" name="es"/>
@@ -8673,6 +8697,14 @@
     <tableColumn id="14" xr3:uid="{2EE64B08-B1B7-D14E-829C-CCCF1AA6F578}" name="ar"/>
     <tableColumn id="15" xr3:uid="{A6FEED21-E84C-D440-959E-4E354BF50866}" name="ru"/>
     <tableColumn id="16" xr3:uid="{99C3C150-8605-BB43-A9F5-712670E10107}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{D844700E-D2CF-7B40-8548-E511FB74A6BC}" name="no"/>
+    <tableColumn id="18" xr3:uid="{821A2492-9EA4-354B-8E2D-740A2153DE3E}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{D697D6CB-0C9D-984E-A606-8A663D311842}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{EB2411D5-EA81-F642-8D13-E8F2128FEE1C}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{DE05A4B3-18D2-A146-A1AB-9E8EB1F63EE0}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{DDE62664-6E47-9842-959E-2FA8C39617C8}" name="el"/>
+    <tableColumn id="23" xr3:uid="{F70C999D-EEFB-D345-8517-DAAB2CA49C4B}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{E38FD840-C043-1740-B0F0-A2C8FFB0CE50}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8701,9 +8733,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4B01E381-89D0-6140-ABAF-45E87900E7A5}" name="Table2" displayName="Table2" ref="A2:P11" totalsRowShown="0">
-  <autoFilter ref="A2:P11" xr:uid="{4B01E381-89D0-6140-ABAF-45E87900E7A5}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4B01E381-89D0-6140-ABAF-45E87900E7A5}" name="Table2" displayName="Table2" ref="A2:X11" totalsRowShown="0">
+  <autoFilter ref="A2:X11" xr:uid="{4B01E381-89D0-6140-ABAF-45E87900E7A5}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{5AE62A60-BB21-4F4F-9CD3-074F4FEE8E6F}" name="key"/>
     <tableColumn id="2" xr3:uid="{9DCC7BEA-4623-AD4C-BFD0-D320033C63F9}" name="en"/>
     <tableColumn id="3" xr3:uid="{7CDC6A0C-D533-D249-946B-9E3A0B92C92D}" name="es"/>
@@ -8720,15 +8752,23 @@
     <tableColumn id="14" xr3:uid="{243142BE-039B-834F-8B3E-75138F791095}" name="ar"/>
     <tableColumn id="15" xr3:uid="{C2D728B1-652C-F04A-92FE-D82B415426EC}" name="ru"/>
     <tableColumn id="16" xr3:uid="{CDE65D78-23BD-8E4E-9F62-4C62A0DF1088}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{96ECF8B0-2B3F-D443-A2D2-A14FA0CDF4C4}" name="no"/>
+    <tableColumn id="18" xr3:uid="{DFED39DF-57C3-984F-AD11-EF6E27E9251B}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{7E318234-EBA4-2A4A-9571-5A6551CF3158}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{74221482-8AC2-A046-95BD-A9B833B916DB}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{F3F1DDD2-E6A9-4C4C-A9A3-451E98013B97}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{C1836C09-D45E-114B-AF94-99C49D7F0B27}" name="el"/>
+    <tableColumn id="23" xr3:uid="{631D1298-27AF-4C49-A23C-3F592A2F4EFC}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{556A5B60-98F3-0247-A1A7-A3DD3249B471}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{58659963-4CE3-6842-AFEF-09BF813541E2}" name="Table3" displayName="Table3" ref="A2:P72" totalsRowShown="0">
-  <autoFilter ref="A2:P72" xr:uid="{58659963-4CE3-6842-AFEF-09BF813541E2}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{58659963-4CE3-6842-AFEF-09BF813541E2}" name="Table3" displayName="Table3" ref="A2:X72" totalsRowShown="0">
+  <autoFilter ref="A2:X72" xr:uid="{58659963-4CE3-6842-AFEF-09BF813541E2}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{D62854E4-9C72-D74F-8C03-E6A8E66842DD}" name="key"/>
     <tableColumn id="2" xr3:uid="{2D9F4322-19AD-BE4F-8D21-50F26FBC17FA}" name="en"/>
     <tableColumn id="3" xr3:uid="{9436FEA3-7677-F84D-AB07-E2EEA95DFADE}" name="es"/>
@@ -8745,15 +8785,23 @@
     <tableColumn id="14" xr3:uid="{FB64AEF9-C278-6B45-8625-6C4A6763FFCB}" name="ar"/>
     <tableColumn id="15" xr3:uid="{055F8455-0748-C743-AE0B-456FF8BC64C7}" name="ru"/>
     <tableColumn id="16" xr3:uid="{0AD9D200-9993-BE49-BC9D-9A754313A134}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{DD2B7F7A-FCF9-7040-85CC-1C11D9601D79}" name="no"/>
+    <tableColumn id="18" xr3:uid="{9F7145FE-FC2F-0040-AAF4-75E2994AA09E}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{F780F4D9-7E5D-1B43-96B7-6A20970622B9}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{AD1A3271-6DED-254C-B77B-28EE6569A951}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{CCBF88E2-C7B4-8F43-AB32-B60F9CB46191}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{7ECB5346-DC9F-D943-8E5C-8DEB16C28CB4}" name="el"/>
+    <tableColumn id="23" xr3:uid="{42CDF424-1DD1-0446-A346-A29A7EF015B9}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{9DFB39DF-3D83-184C-B28F-505A2D8283FF}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7ECF31DB-1F0A-F148-A745-D5CD19B2AAC8}" name="Table4" displayName="Table4" ref="A2:P8" totalsRowShown="0">
-  <autoFilter ref="A2:P8" xr:uid="{7ECF31DB-1F0A-F148-A745-D5CD19B2AAC8}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7ECF31DB-1F0A-F148-A745-D5CD19B2AAC8}" name="Table4" displayName="Table4" ref="A2:X8" totalsRowShown="0">
+  <autoFilter ref="A2:X8" xr:uid="{7ECF31DB-1F0A-F148-A745-D5CD19B2AAC8}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{BB798FA5-2799-7744-B1FC-245269382A01}" name="key"/>
     <tableColumn id="2" xr3:uid="{83076477-6376-2947-817C-8D5B86595D35}" name="en"/>
     <tableColumn id="3" xr3:uid="{55E7B32C-15E3-9944-A7C7-B41A11F9F1C3}" name="es"/>
@@ -8770,15 +8818,23 @@
     <tableColumn id="14" xr3:uid="{9EA482FC-E251-694A-9D10-505EF691AAB3}" name="ar"/>
     <tableColumn id="15" xr3:uid="{109E9DDA-BAA2-F647-AA84-B5806EE323FC}" name="ru"/>
     <tableColumn id="16" xr3:uid="{C6B35678-7862-7544-9920-149295D217F7}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{81109294-1496-9544-9517-B4293B0E7D8E}" name="no"/>
+    <tableColumn id="18" xr3:uid="{35CD2136-CBE0-D744-86A2-61487CB1D1B8}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{9BCEAC8C-0C79-BF46-B6BD-778112D2D50E}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{F72256A5-2739-394C-8BA4-A5789B6A2301}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{C907672D-F76B-2540-83F1-088E8F771C25}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{A641E86A-2212-BB45-AD8F-34FADF5B5BD0}" name="el"/>
+    <tableColumn id="23" xr3:uid="{7C0BC79B-6B23-874B-90B7-A8E8628D6938}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{F47D1C7C-A244-7B42-BE50-66E73EB5B3A1}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0965C627-6E7E-794B-B2F2-551700F896B8}" name="Table5" displayName="Table5" ref="A2:P10" totalsRowShown="0">
-  <autoFilter ref="A2:P10" xr:uid="{0965C627-6E7E-794B-B2F2-551700F896B8}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0965C627-6E7E-794B-B2F2-551700F896B8}" name="Table5" displayName="Table5" ref="A2:X10" totalsRowShown="0">
+  <autoFilter ref="A2:X10" xr:uid="{0965C627-6E7E-794B-B2F2-551700F896B8}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{EE2CB5F7-CC7F-8647-A5B1-D6E43CE4413A}" name="key"/>
     <tableColumn id="2" xr3:uid="{4E90412B-4040-374A-BE7B-FC5D5926CC57}" name="en"/>
     <tableColumn id="3" xr3:uid="{DC5BB12C-67C7-7341-83B1-108FF601E4BF}" name="es"/>
@@ -8795,15 +8851,23 @@
     <tableColumn id="14" xr3:uid="{68281325-04C5-524E-AEF1-49A06CCA5B3A}" name="ar"/>
     <tableColumn id="15" xr3:uid="{207CCBD3-8C1B-874D-99E4-29BAC6AD8DF3}" name="ru"/>
     <tableColumn id="16" xr3:uid="{5665B70F-70AD-3941-8C88-3CAA0F573D1D}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{2B080587-6C47-6641-A6AB-311B88E4D954}" name="no"/>
+    <tableColumn id="18" xr3:uid="{F8599058-6736-D549-AC35-CD90DB181AF9}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{0A163D60-F47B-4B41-9297-2CB8F33AEC08}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{973CBCB8-CA4E-444B-A2BC-CBA6E3608052}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{300F0C51-F271-0541-8880-28F9C5982D09}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{78C291AA-82E0-0445-A3FD-6A0F0A39FFCD}" name="el"/>
+    <tableColumn id="23" xr3:uid="{0906D1B2-42CF-164C-826A-D627C5C1BB95}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{A28F683B-E044-344C-BBA5-3813489F23F6}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E4522DBC-61D7-9C46-8B3A-94857E836847}" name="Table6" displayName="Table6" ref="A2:P6" totalsRowShown="0">
-  <autoFilter ref="A2:P6" xr:uid="{E4522DBC-61D7-9C46-8B3A-94857E836847}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E4522DBC-61D7-9C46-8B3A-94857E836847}" name="Table6" displayName="Table6" ref="A2:X6" totalsRowShown="0">
+  <autoFilter ref="A2:X6" xr:uid="{E4522DBC-61D7-9C46-8B3A-94857E836847}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{75CC3732-2363-C140-9BC5-942207F564D1}" name="key"/>
     <tableColumn id="2" xr3:uid="{994FBB73-3B66-7143-8041-DF75A89266ED}" name="en"/>
     <tableColumn id="3" xr3:uid="{E7FF87A6-CE31-0B4D-82A7-A989A054B211}" name="es"/>
@@ -8820,15 +8884,23 @@
     <tableColumn id="14" xr3:uid="{991ADC19-64BD-1446-9F9C-7494755D5F34}" name="ar"/>
     <tableColumn id="15" xr3:uid="{FB84C9B0-AEE7-554D-8C3B-9253FA43910E}" name="ru"/>
     <tableColumn id="16" xr3:uid="{2E6B1796-7D91-954F-95AC-49B600792D77}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{D0851D8B-398C-6044-8EF3-EE6CA22E714C}" name="no"/>
+    <tableColumn id="18" xr3:uid="{A6206060-280A-F04F-97BB-1C27403F809D}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{3188828F-D62D-AA40-A32B-B6F7F323D967}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{73C6B295-9DD4-CC48-91C4-A9762775EDBC}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{369279A7-1A20-AF4E-A025-211C0A72EF47}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{DFC58A60-89C7-5944-BA0D-BC1B28D27A54}" name="el"/>
+    <tableColumn id="23" xr3:uid="{A09FB64D-7A81-7744-93F3-2AFA201CD06C}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{045F807F-B7DF-2A4B-B883-DA95B3B8DEC6}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AD22473A-E268-8041-82CA-94C2F3C88709}" name="Table7" displayName="Table7" ref="A2:Q4" totalsRowShown="0">
-  <autoFilter ref="A2:Q4" xr:uid="{AD22473A-E268-8041-82CA-94C2F3C88709}"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AD22473A-E268-8041-82CA-94C2F3C88709}" name="Table7" displayName="Table7" ref="A2:Y4" totalsRowShown="0">
+  <autoFilter ref="A2:Y4" xr:uid="{AD22473A-E268-8041-82CA-94C2F3C88709}"/>
+  <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{3232D45D-E159-5242-8B03-876B29C3B6F6}" name="key"/>
     <tableColumn id="2" xr3:uid="{E0467F49-CFD2-424A-BBAB-EE5E103DB67F}" name="en"/>
     <tableColumn id="3" xr3:uid="{B97887F4-5415-DE4B-ACE2-2E7190E4E39C}" name="en_gb"/>
@@ -8846,15 +8918,23 @@
     <tableColumn id="15" xr3:uid="{378AB8A1-C55A-7B47-A0B3-0F888287C530}" name="ar"/>
     <tableColumn id="16" xr3:uid="{46B247E3-8170-FE44-B2DF-A7086B98192B}" name="ru"/>
     <tableColumn id="17" xr3:uid="{AB1D2136-02A1-7045-8225-1578EF14EA2A}" name="tr"/>
+    <tableColumn id="18" xr3:uid="{5AA2BD79-E69A-464B-BE55-827669A98E53}" name="no"/>
+    <tableColumn id="19" xr3:uid="{4FD8C3A9-3411-214E-8B70-1929129BDBB4}" name="sv"/>
+    <tableColumn id="20" xr3:uid="{9AF4C742-D996-C84A-83E3-630947CBEE0E}" name="cs"/>
+    <tableColumn id="21" xr3:uid="{A3EF853A-5D51-5F44-8362-7B3E98682044}" name="hr"/>
+    <tableColumn id="22" xr3:uid="{D2109533-198C-974C-90B1-3F99D1ED45E0}" name="pl"/>
+    <tableColumn id="23" xr3:uid="{F7CEFC49-FF95-F444-BA3C-35DE2465F978}" name="el"/>
+    <tableColumn id="24" xr3:uid="{967CF7CE-8ABA-7B42-899E-87A154242AEB}" name="sw"/>
+    <tableColumn id="25" xr3:uid="{436BAFF6-C49D-934E-ABED-AD046A922524}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{46F0D796-49BE-354C-BAAB-44CE00DA743B}" name="Table8" displayName="Table8" ref="A2:P101" totalsRowShown="0">
-  <autoFilter ref="A2:P101" xr:uid="{46F0D796-49BE-354C-BAAB-44CE00DA743B}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{46F0D796-49BE-354C-BAAB-44CE00DA743B}" name="Table8" displayName="Table8" ref="A2:X101" totalsRowShown="0">
+  <autoFilter ref="A2:X101" xr:uid="{46F0D796-49BE-354C-BAAB-44CE00DA743B}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{3C0114D6-09BB-CA44-8BE7-4646421F7317}" name="key"/>
     <tableColumn id="2" xr3:uid="{170053BE-DDF2-A74A-865B-9970E6229F8E}" name="en"/>
     <tableColumn id="3" xr3:uid="{0FCCB19B-D181-DC4F-8677-CAC3AC92B350}" name="es"/>
@@ -8871,15 +8951,23 @@
     <tableColumn id="14" xr3:uid="{D2B57CE7-A82F-E149-A5EE-397C3A7071DF}" name="ar"/>
     <tableColumn id="15" xr3:uid="{5FEF351A-E40B-B34B-80CA-5BBFCED211CF}" name="ru"/>
     <tableColumn id="16" xr3:uid="{C623C465-BCB8-3949-9F68-197CF23C479E}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{F73E19FC-E16B-2149-8556-5612A2BEA54D}" name="no"/>
+    <tableColumn id="18" xr3:uid="{A15AEED4-2EB1-3548-BF2E-3B85376A5E9F}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{947D118C-BC9F-BC41-80B3-7EE9B857837D}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{ECC5A328-3E8D-264E-ACC7-7A7FB1691DA1}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{0EA86946-351D-1844-B53C-350501406BEA}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{8FD6229F-5524-384D-A91D-BA1FB300ABED}" name="el"/>
+    <tableColumn id="23" xr3:uid="{BE4245BF-65E2-2644-8254-772517EB2FCD}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{8C888E51-14B4-1349-922B-A2B6D78CFC40}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B5648B35-52E8-6247-B3EF-D0550F56A9AD}" name="Table9" displayName="Table9" ref="A2:P43" totalsRowShown="0">
-  <autoFilter ref="A2:P43" xr:uid="{B5648B35-52E8-6247-B3EF-D0550F56A9AD}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B5648B35-52E8-6247-B3EF-D0550F56A9AD}" name="Table9" displayName="Table9" ref="A2:X43" totalsRowShown="0">
+  <autoFilter ref="A2:X43" xr:uid="{B5648B35-52E8-6247-B3EF-D0550F56A9AD}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{F502F998-369B-7647-B58C-8E58430B0958}" name="key"/>
     <tableColumn id="2" xr3:uid="{D332C32F-8E0D-D945-B254-A11E5DC5DCFC}" name="en"/>
     <tableColumn id="3" xr3:uid="{4798F23A-5AFC-6C43-AA7B-C69A3C203E65}" name="es"/>
@@ -8896,6 +8984,14 @@
     <tableColumn id="14" xr3:uid="{BC0758C3-2D2C-1846-A28E-66E91B6C0298}" name="ar"/>
     <tableColumn id="15" xr3:uid="{00F1CC31-5E91-714D-AED8-C87AF78F3CBD}" name="ru"/>
     <tableColumn id="16" xr3:uid="{8C8164AA-1665-B644-8338-DD319599EED0}" name="tr"/>
+    <tableColumn id="17" xr3:uid="{BB67F814-7067-6C4D-890E-F221A4893FEF}" name="no"/>
+    <tableColumn id="18" xr3:uid="{DEC7420B-F5C4-6B4B-BC7A-5DD00D3FB2DC}" name="sv"/>
+    <tableColumn id="19" xr3:uid="{14E0ECFA-25B2-8D43-A2B8-C9B418232FD9}" name="cs"/>
+    <tableColumn id="20" xr3:uid="{E3DE8061-970C-1C4E-A37E-C3B93DF2F07C}" name="hr"/>
+    <tableColumn id="21" xr3:uid="{C800C42E-E9CE-3C47-85A5-A13C1F077B9A}" name="pl"/>
+    <tableColumn id="22" xr3:uid="{3FB3F9CC-64B4-9A43-93D4-CC1A92B804F7}" name="el"/>
+    <tableColumn id="23" xr3:uid="{459C6D7E-54F1-7E4F-AED3-B6BD8292E5B0}" name="sw"/>
+    <tableColumn id="24" xr3:uid="{85D0960F-5C95-EB4F-984F-FE56E82A7FFA}" name="uz"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9186,7 +9282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -9205,7 +9301,7 @@
     <col min="16" max="16" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -9226,8 +9322,9 @@
       <c r="N1" s="3"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="4"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -9276,8 +9373,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -9327,7 +9448,7 @@
         <v>2256</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -9377,7 +9498,7 @@
         <v>2257</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -9412,7 +9533,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -9462,7 +9583,7 @@
         <v>2258</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -10292,7 +10413,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -10311,7 +10432,7 @@
     <col min="16" max="16" width="21.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -10332,8 +10453,9 @@
       <c r="N1" s="3"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="4"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -10382,8 +10504,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>67</v>
       </c>
@@ -10433,7 +10579,7 @@
         <v>2278</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -10483,7 +10629,7 @@
         <v>2279</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>86</v>
       </c>
@@ -10533,7 +10679,7 @@
         <v>2280</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>99</v>
       </c>
@@ -10583,7 +10729,7 @@
         <v>2281</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>109</v>
       </c>
@@ -10633,7 +10779,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>118</v>
       </c>
@@ -10683,7 +10829,7 @@
         <v>2282</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>128</v>
       </c>
@@ -10733,7 +10879,7 @@
         <v>2283</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -10783,7 +10929,7 @@
         <v>2284</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>151</v>
       </c>
@@ -10844,7 +10990,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:X72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -10862,7 +11008,7 @@
     <col min="16" max="16" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -10883,8 +11029,9 @@
       <c r="N1" s="3"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="4"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -10933,8 +11080,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>163</v>
       </c>
@@ -10984,7 +11155,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>172</v>
       </c>
@@ -11034,7 +11205,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>179</v>
       </c>
@@ -11084,7 +11255,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>186</v>
       </c>
@@ -11134,7 +11305,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>192</v>
       </c>
@@ -11184,7 +11355,7 @@
         <v>2765</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>200</v>
       </c>
@@ -11234,7 +11405,7 @@
         <v>2766</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>210</v>
       </c>
@@ -11284,7 +11455,7 @@
         <v>2767</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>217</v>
       </c>
@@ -11334,7 +11505,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>224</v>
       </c>
@@ -11384,7 +11555,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>231</v>
       </c>
@@ -11434,7 +11605,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>241</v>
       </c>
@@ -11484,7 +11655,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>251</v>
       </c>
@@ -11534,7 +11705,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>257</v>
       </c>
@@ -11584,7 +11755,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>264</v>
       </c>
@@ -14445,7 +14616,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -14456,7 +14627,7 @@
     <col min="16" max="16" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -14477,8 +14648,9 @@
       <c r="N1" s="3"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="4"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -14527,8 +14699,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>719</v>
       </c>
@@ -14578,7 +14774,7 @@
         <v>2408</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>732</v>
       </c>
@@ -14586,7 +14782,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>734</v>
       </c>
@@ -14600,7 +14796,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>737</v>
       </c>
@@ -14650,7 +14846,7 @@
         <v>2409</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>749</v>
       </c>
@@ -14700,7 +14896,7 @@
         <v>2410</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>760</v>
       </c>
@@ -14740,7 +14936,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -14759,7 +14955,7 @@
     <col min="16" max="16" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -14781,7 +14977,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -14830,8 +15026,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>764</v>
       </c>
@@ -14881,7 +15101,7 @@
         <v>2427</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>776</v>
       </c>
@@ -14931,7 +15151,7 @@
         <v>2428</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>789</v>
       </c>
@@ -14981,7 +15201,7 @@
         <v>2429</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>796</v>
       </c>
@@ -15031,7 +15251,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>807</v>
       </c>
@@ -15081,7 +15301,7 @@
         <v>2431</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>819</v>
       </c>
@@ -15131,7 +15351,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>832</v>
       </c>
@@ -15181,7 +15401,7 @@
         <v>2433</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>845</v>
       </c>
@@ -15242,7 +15462,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:X6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" bestFit="1" customWidth="1"/>
@@ -15259,7 +15479,7 @@
     <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -15281,7 +15501,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -15330,8 +15550,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>854</v>
       </c>
@@ -15381,7 +15625,7 @@
         <v>2442</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>866</v>
       </c>
@@ -15431,7 +15675,7 @@
         <v>2443</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>876</v>
       </c>
@@ -15481,7 +15725,7 @@
         <v>2444</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>884</v>
       </c>
@@ -15542,7 +15786,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -15560,7 +15804,7 @@
     <col min="17" max="17" width="6.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -15583,7 +15827,7 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -15635,8 +15879,32 @@
       <c r="Q2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>892</v>
       </c>
@@ -15689,7 +15957,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>902</v>
       </c>
@@ -15750,7 +16018,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:X101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
@@ -15771,7 +16039,7 @@
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -15793,7 +16061,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -15842,8 +16110,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>913</v>
       </c>
@@ -15893,7 +16185,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>923</v>
       </c>
@@ -15943,7 +16235,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>933</v>
       </c>
@@ -15993,7 +16285,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>943</v>
       </c>
@@ -16043,7 +16335,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>953</v>
       </c>
@@ -16093,7 +16385,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>963</v>
       </c>
@@ -16143,7 +16435,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>973</v>
       </c>
@@ -16193,7 +16485,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>983</v>
       </c>
@@ -16243,7 +16535,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>993</v>
       </c>
@@ -16293,7 +16585,7 @@
         <v>2633</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1004</v>
       </c>
@@ -16343,7 +16635,7 @@
         <v>2634</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>1016</v>
       </c>
@@ -16393,7 +16685,7 @@
         <v>2635</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>1025</v>
       </c>
@@ -16443,7 +16735,7 @@
         <v>2636</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>1036</v>
       </c>
@@ -16493,7 +16785,7 @@
         <v>2637</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1046</v>
       </c>
@@ -20804,7 +21096,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:X43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
@@ -20825,7 +21117,7 @@
     <col min="18" max="18" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2222</v>
       </c>
@@ -20847,7 +21139,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -20896,8 +21188,32 @@
       <c r="P2" t="s">
         <v>2252</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>2810</v>
+      </c>
+      <c r="R2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="T2" t="s">
+        <v>2813</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2814</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2809</v>
+      </c>
+      <c r="W2" t="s">
+        <v>2815</v>
+      </c>
+      <c r="X2" t="s">
+        <v>2816</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1873</v>
       </c>
@@ -20947,7 +21263,7 @@
         <v>1874</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1654</v>
       </c>
@@ -20997,7 +21313,7 @@
         <v>1880</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1887</v>
       </c>
@@ -21047,7 +21363,7 @@
         <v>2760</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1894</v>
       </c>
@@ -21097,7 +21413,7 @@
         <v>1895</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1902</v>
       </c>
@@ -21147,7 +21463,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1911</v>
       </c>
@@ -21197,7 +21513,7 @@
         <v>1912</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>1920</v>
       </c>
@@ -21247,7 +21563,7 @@
         <v>1921</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1926</v>
       </c>
@@ -21297,7 +21613,7 @@
         <v>1927</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>1938</v>
       </c>
@@ -21347,7 +21663,7 @@
         <v>2761</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1948</v>
       </c>
@@ -21397,7 +21713,7 @@
         <v>1949</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>1960</v>
       </c>
@@ -21447,7 +21763,7 @@
         <v>1961</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>1967</v>
       </c>
@@ -21497,7 +21813,7 @@
         <v>1968</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>1973</v>
       </c>
@@ -21547,7 +21863,7 @@
         <v>1974</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1981</v>
       </c>

</xml_diff>

<commit_message>
norwegian language code: nb not no
</commit_message>
<xml_diff>
--- a/src/stp/database/localization.xlsx
+++ b/src/stp/database/localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35486CF-AEDC-B046-9067-639E827FE6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30EFEE51-7D7A-6040-979E-FA3A0821E168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Competition" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4328" uniqueCount="2817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4328" uniqueCount="2818">
   <si>
     <t>key</t>
   </si>
@@ -8480,6 +8480,9 @@
   </si>
   <si>
     <t>uz</t>
+  </si>
+  <si>
+    <t>nb</t>
   </si>
 </sst>
 </file>
@@ -8697,7 +8700,7 @@
     <tableColumn id="14" xr3:uid="{2EE64B08-B1B7-D14E-829C-CCCF1AA6F578}" name="ar"/>
     <tableColumn id="15" xr3:uid="{A6FEED21-E84C-D440-959E-4E354BF50866}" name="ru"/>
     <tableColumn id="16" xr3:uid="{99C3C150-8605-BB43-A9F5-712670E10107}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{D844700E-D2CF-7B40-8548-E511FB74A6BC}" name="no"/>
+    <tableColumn id="17" xr3:uid="{D844700E-D2CF-7B40-8548-E511FB74A6BC}" name="nb"/>
     <tableColumn id="18" xr3:uid="{821A2492-9EA4-354B-8E2D-740A2153DE3E}" name="sv"/>
     <tableColumn id="19" xr3:uid="{D697D6CB-0C9D-984E-A606-8A663D311842}" name="cs"/>
     <tableColumn id="20" xr3:uid="{EB2411D5-EA81-F642-8D13-E8F2128FEE1C}" name="hr"/>
@@ -8785,7 +8788,7 @@
     <tableColumn id="14" xr3:uid="{FB64AEF9-C278-6B45-8625-6C4A6763FFCB}" name="ar"/>
     <tableColumn id="15" xr3:uid="{055F8455-0748-C743-AE0B-456FF8BC64C7}" name="ru"/>
     <tableColumn id="16" xr3:uid="{0AD9D200-9993-BE49-BC9D-9A754313A134}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{DD2B7F7A-FCF9-7040-85CC-1C11D9601D79}" name="no"/>
+    <tableColumn id="17" xr3:uid="{DD2B7F7A-FCF9-7040-85CC-1C11D9601D79}" name="nb"/>
     <tableColumn id="18" xr3:uid="{9F7145FE-FC2F-0040-AAF4-75E2994AA09E}" name="sv"/>
     <tableColumn id="19" xr3:uid="{F780F4D9-7E5D-1B43-96B7-6A20970622B9}" name="cs"/>
     <tableColumn id="20" xr3:uid="{AD1A3271-6DED-254C-B77B-28EE6569A951}" name="hr"/>
@@ -8818,7 +8821,7 @@
     <tableColumn id="14" xr3:uid="{9EA482FC-E251-694A-9D10-505EF691AAB3}" name="ar"/>
     <tableColumn id="15" xr3:uid="{109E9DDA-BAA2-F647-AA84-B5806EE323FC}" name="ru"/>
     <tableColumn id="16" xr3:uid="{C6B35678-7862-7544-9920-149295D217F7}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{81109294-1496-9544-9517-B4293B0E7D8E}" name="no"/>
+    <tableColumn id="17" xr3:uid="{81109294-1496-9544-9517-B4293B0E7D8E}" name="nb"/>
     <tableColumn id="18" xr3:uid="{35CD2136-CBE0-D744-86A2-61487CB1D1B8}" name="sv"/>
     <tableColumn id="19" xr3:uid="{9BCEAC8C-0C79-BF46-B6BD-778112D2D50E}" name="cs"/>
     <tableColumn id="20" xr3:uid="{F72256A5-2739-394C-8BA4-A5789B6A2301}" name="hr"/>
@@ -8851,7 +8854,7 @@
     <tableColumn id="14" xr3:uid="{68281325-04C5-524E-AEF1-49A06CCA5B3A}" name="ar"/>
     <tableColumn id="15" xr3:uid="{207CCBD3-8C1B-874D-99E4-29BAC6AD8DF3}" name="ru"/>
     <tableColumn id="16" xr3:uid="{5665B70F-70AD-3941-8C88-3CAA0F573D1D}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{2B080587-6C47-6641-A6AB-311B88E4D954}" name="no"/>
+    <tableColumn id="17" xr3:uid="{2B080587-6C47-6641-A6AB-311B88E4D954}" name="nb"/>
     <tableColumn id="18" xr3:uid="{F8599058-6736-D549-AC35-CD90DB181AF9}" name="sv"/>
     <tableColumn id="19" xr3:uid="{0A163D60-F47B-4B41-9297-2CB8F33AEC08}" name="cs"/>
     <tableColumn id="20" xr3:uid="{973CBCB8-CA4E-444B-A2BC-CBA6E3608052}" name="hr"/>
@@ -8884,7 +8887,7 @@
     <tableColumn id="14" xr3:uid="{991ADC19-64BD-1446-9F9C-7494755D5F34}" name="ar"/>
     <tableColumn id="15" xr3:uid="{FB84C9B0-AEE7-554D-8C3B-9253FA43910E}" name="ru"/>
     <tableColumn id="16" xr3:uid="{2E6B1796-7D91-954F-95AC-49B600792D77}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{D0851D8B-398C-6044-8EF3-EE6CA22E714C}" name="no"/>
+    <tableColumn id="17" xr3:uid="{D0851D8B-398C-6044-8EF3-EE6CA22E714C}" name="nb"/>
     <tableColumn id="18" xr3:uid="{A6206060-280A-F04F-97BB-1C27403F809D}" name="sv"/>
     <tableColumn id="19" xr3:uid="{3188828F-D62D-AA40-A32B-B6F7F323D967}" name="cs"/>
     <tableColumn id="20" xr3:uid="{73C6B295-9DD4-CC48-91C4-A9762775EDBC}" name="hr"/>
@@ -8918,7 +8921,7 @@
     <tableColumn id="15" xr3:uid="{378AB8A1-C55A-7B47-A0B3-0F888287C530}" name="ar"/>
     <tableColumn id="16" xr3:uid="{46B247E3-8170-FE44-B2DF-A7086B98192B}" name="ru"/>
     <tableColumn id="17" xr3:uid="{AB1D2136-02A1-7045-8225-1578EF14EA2A}" name="tr"/>
-    <tableColumn id="18" xr3:uid="{5AA2BD79-E69A-464B-BE55-827669A98E53}" name="no"/>
+    <tableColumn id="18" xr3:uid="{5AA2BD79-E69A-464B-BE55-827669A98E53}" name="nb"/>
     <tableColumn id="19" xr3:uid="{4FD8C3A9-3411-214E-8B70-1929129BDBB4}" name="sv"/>
     <tableColumn id="20" xr3:uid="{9AF4C742-D996-C84A-83E3-630947CBEE0E}" name="cs"/>
     <tableColumn id="21" xr3:uid="{A3EF853A-5D51-5F44-8362-7B3E98682044}" name="hr"/>
@@ -8951,7 +8954,7 @@
     <tableColumn id="14" xr3:uid="{D2B57CE7-A82F-E149-A5EE-397C3A7071DF}" name="ar"/>
     <tableColumn id="15" xr3:uid="{5FEF351A-E40B-B34B-80CA-5BBFCED211CF}" name="ru"/>
     <tableColumn id="16" xr3:uid="{C623C465-BCB8-3949-9F68-197CF23C479E}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{F73E19FC-E16B-2149-8556-5612A2BEA54D}" name="no"/>
+    <tableColumn id="17" xr3:uid="{F73E19FC-E16B-2149-8556-5612A2BEA54D}" name="nb"/>
     <tableColumn id="18" xr3:uid="{A15AEED4-2EB1-3548-BF2E-3B85376A5E9F}" name="sv"/>
     <tableColumn id="19" xr3:uid="{947D118C-BC9F-BC41-80B3-7EE9B857837D}" name="cs"/>
     <tableColumn id="20" xr3:uid="{ECC5A328-3E8D-264E-ACC7-7A7FB1691DA1}" name="hr"/>
@@ -8984,7 +8987,7 @@
     <tableColumn id="14" xr3:uid="{BC0758C3-2D2C-1846-A28E-66E91B6C0298}" name="ar"/>
     <tableColumn id="15" xr3:uid="{00F1CC31-5E91-714D-AED8-C87AF78F3CBD}" name="ru"/>
     <tableColumn id="16" xr3:uid="{8C8164AA-1665-B644-8338-DD319599EED0}" name="tr"/>
-    <tableColumn id="17" xr3:uid="{BB67F814-7067-6C4D-890E-F221A4893FEF}" name="no"/>
+    <tableColumn id="17" xr3:uid="{BB67F814-7067-6C4D-890E-F221A4893FEF}" name="nb"/>
     <tableColumn id="18" xr3:uid="{DEC7420B-F5C4-6B4B-BC7A-5DD00D3FB2DC}" name="sv"/>
     <tableColumn id="19" xr3:uid="{14E0ECFA-25B2-8D43-A2B8-C9B418232FD9}" name="cs"/>
     <tableColumn id="20" xr3:uid="{E3DE8061-970C-1C4E-A37E-C3B93DF2F07C}" name="hr"/>
@@ -9374,7 +9377,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -11081,7 +11084,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -14700,7 +14703,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -15027,7 +15030,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -15551,7 +15554,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -15880,7 +15883,7 @@
         <v>2252</v>
       </c>
       <c r="R2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="S2" t="s">
         <v>2811</v>
@@ -16111,7 +16114,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>
@@ -21189,7 +21192,7 @@
         <v>2252</v>
       </c>
       <c r="Q2" t="s">
-        <v>2810</v>
+        <v>2817</v>
       </c>
       <c r="R2" t="s">
         <v>2811</v>

</xml_diff>